<commit_message>
new pages with dynamic csv
clausulas vencidas se lee dinamicamente de un csv generado automaticamente por el dashboard de clausulas
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg.sharepoint.com/sites/CIDCCR_CIDCCR_EquipoOperaciones/Shared Documents/General/torre de control/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D328ECC4-DFF5-404B-8118-6876A08204F0}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50726C49-A423-423D-AC6D-B4556D156766}"/>
   <bookViews>
-    <workbookView xWindow="756" yWindow="48" windowWidth="21528" windowHeight="13188" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7920" yWindow="1320" windowWidth="19275" windowHeight="13800" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="documentos" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="clausulas 180 dias" sheetId="4" r:id="rId4"/>
     <sheet name="productos criticos" sheetId="5" r:id="rId5"/>
     <sheet name="PMR" sheetId="6" r:id="rId6"/>
-    <sheet name="change log" sheetId="7" r:id="rId7"/>
-    <sheet name="datos_ops" sheetId="8" r:id="rId8"/>
+    <sheet name="datos_ops" sheetId="8" r:id="rId7"/>
+    <sheet name="change log" sheetId="7" r:id="rId8"/>
+    <sheet name="Sheet2" sheetId="10" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'clausulas 180 dias'!$B$4:$K$13</definedName>
@@ -1925,7 +1926,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2147,55 +2148,43 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
@@ -2533,25 +2522,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D59"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="66" customWidth="1"/>
     <col min="2" max="2" width="38" style="66" customWidth="1"/>
     <col min="3" max="3" width="42" style="66" customWidth="1"/>
     <col min="4" max="4" width="80" style="66" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="66"/>
+    <col min="5" max="16384" width="8.85546875" style="66"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="77" t="s">
+    <row r="1" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-    </row>
-    <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+    </row>
+    <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="67" t="s">
         <v>1</v>
       </c>
@@ -2565,7 +2554,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="67" t="s">
         <v>5</v>
       </c>
@@ -2579,7 +2568,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="67" t="s">
         <v>5</v>
       </c>
@@ -2593,7 +2582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="67" t="s">
         <v>11</v>
       </c>
@@ -2607,7 +2596,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="67" t="s">
         <v>14</v>
       </c>
@@ -2621,7 +2610,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="67" t="s">
         <v>17</v>
       </c>
@@ -2635,7 +2624,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="67" t="s">
         <v>20</v>
       </c>
@@ -2649,7 +2638,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="67" t="s">
         <v>22</v>
       </c>
@@ -2663,7 +2652,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="67" t="s">
         <v>25</v>
       </c>
@@ -2677,7 +2666,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="67" t="s">
         <v>5</v>
       </c>
@@ -2691,7 +2680,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="67" t="s">
         <v>14</v>
       </c>
@@ -2705,7 +2694,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="67" t="s">
         <v>17</v>
       </c>
@@ -2719,7 +2708,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
         <v>20</v>
       </c>
@@ -2733,7 +2722,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="67" t="s">
         <v>22</v>
       </c>
@@ -2747,7 +2736,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
         <v>25</v>
       </c>
@@ -2761,7 +2750,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="67" t="s">
         <v>41</v>
       </c>
@@ -2773,7 +2762,7 @@
       </c>
       <c r="D18" s="68"/>
     </row>
-    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="67" t="s">
         <v>5</v>
       </c>
@@ -2787,7 +2776,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="67" t="s">
         <v>11</v>
       </c>
@@ -2801,7 +2790,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="67" t="s">
         <v>14</v>
       </c>
@@ -2815,7 +2804,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="67" t="s">
         <v>17</v>
       </c>
@@ -2829,7 +2818,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="67" t="s">
         <v>20</v>
       </c>
@@ -2843,7 +2832,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="67" t="s">
         <v>22</v>
       </c>
@@ -2857,7 +2846,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="67" t="s">
         <v>25</v>
       </c>
@@ -2871,7 +2860,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="67" t="s">
         <v>58</v>
       </c>
@@ -2885,7 +2874,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="67" t="s">
         <v>5</v>
       </c>
@@ -2899,7 +2888,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="67" t="s">
         <v>14</v>
       </c>
@@ -2913,7 +2902,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="67" t="s">
         <v>17</v>
       </c>
@@ -2927,7 +2916,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="67" t="s">
         <v>20</v>
       </c>
@@ -2941,7 +2930,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="67" t="s">
         <v>22</v>
       </c>
@@ -2955,7 +2944,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="67" t="s">
         <v>41</v>
       </c>
@@ -2969,7 +2958,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="67" t="s">
         <v>58</v>
       </c>
@@ -2983,7 +2972,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="67" t="s">
         <v>5</v>
       </c>
@@ -2997,7 +2986,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="67" t="s">
         <v>5</v>
       </c>
@@ -3011,7 +3000,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="67" t="s">
         <v>11</v>
       </c>
@@ -3025,7 +3014,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="67" t="s">
         <v>14</v>
       </c>
@@ -3039,7 +3028,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="67" t="s">
         <v>17</v>
       </c>
@@ -3053,7 +3042,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="67" t="s">
         <v>20</v>
       </c>
@@ -3067,7 +3056,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="67" t="s">
         <v>22</v>
       </c>
@@ -3081,7 +3070,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="67" t="s">
         <v>25</v>
       </c>
@@ -3095,7 +3084,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="67" t="s">
         <v>58</v>
       </c>
@@ -3109,7 +3098,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="67" t="s">
         <v>5</v>
       </c>
@@ -3123,7 +3112,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="67" t="s">
         <v>14</v>
       </c>
@@ -3137,7 +3126,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="67" t="s">
         <v>17</v>
       </c>
@@ -3151,7 +3140,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="67" t="s">
         <v>20</v>
       </c>
@@ -3165,7 +3154,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="67" t="s">
         <v>58</v>
       </c>
@@ -3179,7 +3168,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="67" t="s">
         <v>5</v>
       </c>
@@ -3193,7 +3182,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="67" t="s">
         <v>11</v>
       </c>
@@ -3207,7 +3196,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="67" t="s">
         <v>14</v>
       </c>
@@ -3221,7 +3210,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="67" t="s">
         <v>17</v>
       </c>
@@ -3235,7 +3224,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="67" t="s">
         <v>20</v>
       </c>
@@ -3249,7 +3238,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="67" t="s">
         <v>22</v>
       </c>
@@ -3263,7 +3252,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="67" t="s">
         <v>25</v>
       </c>
@@ -3277,7 +3266,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="67" t="s">
         <v>5</v>
       </c>
@@ -3291,7 +3280,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="67" t="s">
         <v>11</v>
       </c>
@@ -3303,7 +3292,7 @@
       </c>
       <c r="D56" s="68"/>
     </row>
-    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="67" t="s">
         <v>17</v>
       </c>
@@ -3317,7 +3306,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="67" t="s">
         <v>20</v>
       </c>
@@ -3331,7 +3320,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="67" t="s">
         <v>25</v>
       </c>
@@ -3355,31 +3344,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:K21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.5546875" customWidth="1"/>
-    <col min="3" max="3" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" customWidth="1"/>
+    <col min="3" max="3" width="35.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6">
         <v>46162</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>128</v>
       </c>
@@ -3411,7 +3400,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>129</v>
       </c>
@@ -3443,7 +3432,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>135</v>
       </c>
@@ -3475,7 +3464,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>135</v>
       </c>
@@ -3491,7 +3480,7 @@
       </c>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>142</v>
       </c>
@@ -3521,7 +3510,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>146</v>
       </c>
@@ -3543,7 +3532,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>148</v>
       </c>
@@ -3575,7 +3564,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>150</v>
       </c>
@@ -3607,7 +3596,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>152</v>
       </c>
@@ -3639,7 +3628,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>154</v>
       </c>
@@ -3669,7 +3658,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>154</v>
       </c>
@@ -3693,7 +3682,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
         <v>159</v>
       </c>
@@ -3725,7 +3714,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>162</v>
       </c>
@@ -3757,7 +3746,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>166</v>
       </c>
@@ -3785,7 +3774,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
         <v>168</v>
       </c>
@@ -3807,7 +3796,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
         <v>170</v>
       </c>
@@ -3825,7 +3814,7 @@
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>171</v>
       </c>
@@ -3849,28 +3838,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.44140625" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="5" width="11.6640625" customWidth="1"/>
-    <col min="9" max="9" width="45.44140625" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" customWidth="1"/>
-    <col min="11" max="11" width="44.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="5" width="11.7109375" customWidth="1"/>
+    <col min="9" max="9" width="45.42578125" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
+    <col min="11" max="11" width="44.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6">
         <v>46160</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>172</v>
       </c>
@@ -3902,7 +3891,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="9">
         <v>670362</v>
       </c>
@@ -3934,7 +3923,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
         <v>664364</v>
       </c>
@@ -3964,7 +3953,7 @@
       </c>
       <c r="K6" s="10"/>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
         <v>705321</v>
       </c>
@@ -3994,7 +3983,7 @@
       </c>
       <c r="K7" s="10"/>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="9">
         <v>705320</v>
       </c>
@@ -4024,7 +4013,7 @@
       </c>
       <c r="K8" s="10"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="9">
         <v>690057</v>
       </c>
@@ -4056,7 +4045,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="9">
         <v>690057</v>
       </c>
@@ -4088,7 +4077,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="9">
         <v>701800</v>
       </c>
@@ -4120,7 +4109,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="9">
         <v>692690</v>
       </c>
@@ -4152,7 +4141,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:11" ht="24" x14ac:dyDescent="0.25">
       <c r="B13" s="9">
         <v>701558</v>
       </c>
@@ -4182,7 +4171,7 @@
       </c>
       <c r="K13" s="10"/>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="9">
         <v>687164</v>
       </c>
@@ -4223,31 +4212,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:K15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
     <col min="6" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
-    <col min="9" max="9" width="28.6640625" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6">
         <v>46160</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:11" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>172</v>
       </c>
@@ -4279,7 +4268,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="10">
         <v>692694</v>
       </c>
@@ -4309,10 +4298,10 @@
       </c>
       <c r="K5" s="10">
         <f t="shared" ref="K5:K13" ca="1" si="0">J5-TODAY()</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="10">
         <v>701797</v>
       </c>
@@ -4342,10 +4331,10 @@
       </c>
       <c r="K6" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="10">
         <v>691923</v>
       </c>
@@ -4375,10 +4364,10 @@
       </c>
       <c r="K7" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="10">
         <v>691920</v>
       </c>
@@ -4408,10 +4397,10 @@
       </c>
       <c r="K8" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="10">
         <v>692683</v>
       </c>
@@ -4441,10 +4430,10 @@
       </c>
       <c r="K9" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10">
         <v>701675</v>
       </c>
@@ -4474,10 +4463,10 @@
       </c>
       <c r="K10" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>114</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11" ht="24" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="24" x14ac:dyDescent="0.25">
       <c r="B11" s="10">
         <v>664339</v>
       </c>
@@ -4507,10 +4496,10 @@
       </c>
       <c r="K11" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="10">
         <v>191156</v>
       </c>
@@ -4540,10 +4529,10 @@
       </c>
       <c r="K12" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="10">
         <v>191155</v>
       </c>
@@ -4573,10 +4562,10 @@
       </c>
       <c r="K13" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>171</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11" ht="24" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" ht="24" x14ac:dyDescent="0.25">
       <c r="B14" s="10">
         <v>701540</v>
       </c>
@@ -4606,10 +4595,10 @@
       </c>
       <c r="K14" s="10">
         <f t="shared" ref="K14:K15" ca="1" si="1">J14-TODAY()</f>
-        <v>98</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="10">
         <v>701557</v>
       </c>
@@ -4639,7 +4628,7 @@
       </c>
       <c r="K15" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -4656,25 +4645,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:G41"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="39.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="37.109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="69.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="2"/>
+    <col min="3" max="3" width="46.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="39.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="37.140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="69.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="43" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>218</v>
       </c>
@@ -4694,7 +4683,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="17" t="s">
         <v>17</v>
       </c>
@@ -4710,7 +4699,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="22" t="s">
         <v>17</v>
       </c>
@@ -4724,7 +4713,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="22" t="s">
         <v>17</v>
       </c>
@@ -4744,7 +4733,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="22" t="s">
         <v>17</v>
       </c>
@@ -4764,7 +4753,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="27" t="s">
         <v>17</v>
       </c>
@@ -4780,7 +4769,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="22" t="s">
         <v>17</v>
       </c>
@@ -4794,7 +4783,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="22" t="s">
         <v>17</v>
       </c>
@@ -4814,7 +4803,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="58.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" ht="58.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="32" t="s">
         <v>17</v>
       </c>
@@ -4830,7 +4819,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="17" t="s">
         <v>22</v>
       </c>
@@ -4850,7 +4839,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="32" t="s">
         <v>22</v>
       </c>
@@ -4870,7 +4859,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="38" t="s">
         <v>22</v>
       </c>
@@ -4890,7 +4879,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="17" t="s">
         <v>22</v>
       </c>
@@ -4910,7 +4899,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="22" t="s">
         <v>22</v>
       </c>
@@ -4927,7 +4916,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="32" t="s">
         <v>22</v>
       </c>
@@ -4945,7 +4934,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="137.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="137.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="17" t="s">
         <v>25</v>
       </c>
@@ -4965,23 +4954,23 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="137.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" ht="137.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="81" t="s">
+      <c r="C19" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="D19" s="84" t="s">
+      <c r="D19" s="26" t="s">
         <v>429</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>430</v>
       </c>
-      <c r="F19" s="83"/>
+      <c r="F19" s="23"/>
       <c r="G19" s="25"/>
     </row>
-    <row r="20" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="22" t="s">
         <v>25</v>
       </c>
@@ -5001,7 +4990,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="22" t="s">
         <v>25</v>
       </c>
@@ -5015,10 +5004,10 @@
         <v>433</v>
       </c>
       <c r="F21" s="23"/>
-      <c r="G21" s="83"/>
-    </row>
-    <row r="22" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="85" t="s">
+      <c r="G21" s="23"/>
+    </row>
+    <row r="22" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="77" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="30" t="s">
@@ -5031,137 +5020,132 @@
         <v>264</v>
       </c>
       <c r="F22" s="30"/>
-      <c r="G22" s="86"/>
-    </row>
-    <row r="23" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="87" t="s">
+      <c r="G22" s="78"/>
+    </row>
+    <row r="23" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="81" t="s">
+      <c r="C23" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="D23" s="82" t="s">
+      <c r="D23" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E23" s="83"/>
-      <c r="F23" s="81"/>
-      <c r="G23" s="88"/>
-    </row>
-    <row r="24" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="87" t="s">
+      <c r="E23" s="23"/>
+      <c r="G23" s="80"/>
+    </row>
+    <row r="24" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="81" t="s">
+      <c r="C24" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="D24" s="82" t="s">
+      <c r="D24" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E24" s="83"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="88"/>
-    </row>
-    <row r="25" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="87" t="s">
+      <c r="E24" s="23"/>
+      <c r="G24" s="80"/>
+    </row>
+    <row r="25" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="81" t="s">
+      <c r="C25" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="D25" s="82" t="s">
+      <c r="D25" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E25" s="83"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="88"/>
-    </row>
-    <row r="26" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="87" t="s">
+      <c r="E25" s="23"/>
+      <c r="G25" s="80"/>
+    </row>
+    <row r="26" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="81" t="s">
+      <c r="C26" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="D26" s="82" t="s">
+      <c r="D26" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E26" s="83"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="88"/>
-    </row>
-    <row r="27" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="87" t="s">
+      <c r="E26" s="23"/>
+      <c r="G26" s="80"/>
+    </row>
+    <row r="27" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C27" s="81" t="s">
+      <c r="C27" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="D27" s="82" t="s">
+      <c r="D27" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E27" s="83"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="88"/>
-    </row>
-    <row r="28" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="87" t="s">
+      <c r="E27" s="23"/>
+      <c r="G27" s="80"/>
+    </row>
+    <row r="28" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="81" t="s">
+      <c r="C28" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="D28" s="82" t="s">
+      <c r="D28" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="E28" s="83" t="s">
+      <c r="E28" s="23" t="s">
         <v>420</v>
       </c>
-      <c r="F28" s="83" t="s">
+      <c r="F28" s="23" t="s">
         <v>427</v>
       </c>
-      <c r="G28" s="88"/>
-    </row>
-    <row r="29" spans="2:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="89" t="s">
+      <c r="G28" s="80"/>
+    </row>
+    <row r="29" spans="2:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="81" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="90" t="s">
+      <c r="C29" s="82" t="s">
         <v>417</v>
       </c>
-      <c r="D29" s="91" t="s">
+      <c r="D29" s="83" t="s">
         <v>228</v>
       </c>
-      <c r="E29" s="92" t="s">
+      <c r="E29" s="84" t="s">
         <v>418</v>
       </c>
-      <c r="F29" s="83" t="s">
+      <c r="F29" s="23" t="s">
         <v>427</v>
       </c>
-      <c r="G29" s="93" t="s">
+      <c r="G29" s="85" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="99" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C30" s="83" t="s">
+      <c r="C30" s="23" t="s">
         <v>266</v>
       </c>
-      <c r="D30" s="84" t="s">
+      <c r="D30" s="26" t="s">
         <v>230</v>
       </c>
-      <c r="E30" s="81" t="s">
+      <c r="E30" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="F30" s="83" t="s">
+      <c r="F30" s="23" t="s">
         <v>268</v>
       </c>
       <c r="G30" s="25" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="22" t="s">
         <v>20</v>
       </c>
@@ -5181,7 +5165,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="104.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="22" t="s">
         <v>20</v>
       </c>
@@ -5201,7 +5185,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="22" t="s">
         <v>20</v>
       </c>
@@ -5221,7 +5205,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="17" t="s">
         <v>279</v>
       </c>
@@ -5234,14 +5218,14 @@
       <c r="E34" s="18" t="s">
         <v>281</v>
       </c>
-      <c r="F34" s="79" t="s">
+      <c r="F34" s="86" t="s">
         <v>282</v>
       </c>
       <c r="G34" s="21" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="22" t="s">
         <v>279</v>
       </c>
@@ -5254,12 +5238,12 @@
       <c r="E35" s="23" t="s">
         <v>285</v>
       </c>
-      <c r="F35" s="80"/>
+      <c r="F35" s="87"/>
       <c r="G35" s="25" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:7" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="22" t="s">
         <v>279</v>
       </c>
@@ -5272,12 +5256,12 @@
       <c r="E36" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="F36" s="80"/>
+      <c r="F36" s="87"/>
       <c r="G36" s="25" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="195" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" ht="195" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="17" t="s">
         <v>5</v>
       </c>
@@ -5297,7 +5281,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" ht="188.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="22" t="s">
         <v>5</v>
       </c>
@@ -5317,7 +5301,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="22" t="s">
         <v>5</v>
       </c>
@@ -5337,7 +5321,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="22" t="s">
         <v>5</v>
       </c>
@@ -5354,7 +5338,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:7" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="32" t="s">
         <v>5</v>
       </c>
@@ -5384,29 +5368,29 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:Q14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="57.109375" customWidth="1"/>
-    <col min="4" max="5" width="19.33203125" customWidth="1"/>
+    <col min="3" max="3" width="57.140625" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="9.88671875" customWidth="1"/>
-    <col min="10" max="11" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="7.88671875" customWidth="1"/>
-    <col min="13" max="13" width="62.44140625" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" customWidth="1"/>
+    <col min="10" max="11" width="10.5703125" customWidth="1"/>
+    <col min="12" max="12" width="7.85546875" customWidth="1"/>
+    <col min="13" max="13" width="62.42578125" customWidth="1"/>
     <col min="14" max="14" width="45" customWidth="1"/>
-    <col min="16" max="17" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="65" t="s">
         <v>303</v>
       </c>
       <c r="C2" s="65"/>
     </row>
-    <row r="4" spans="2:17" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="75" t="s">
         <v>174</v>
       </c>
@@ -5447,7 +5431,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="76" t="s">
         <v>5</v>
       </c>
@@ -5488,7 +5472,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="76" t="s">
         <v>11</v>
       </c>
@@ -5529,7 +5513,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="76" t="s">
         <v>20</v>
       </c>
@@ -5570,7 +5554,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="76" t="s">
         <v>25</v>
       </c>
@@ -5611,7 +5595,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="76" t="s">
         <v>17</v>
       </c>
@@ -5652,7 +5636,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="76" t="s">
         <v>22</v>
       </c>
@@ -5693,7 +5677,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="76" t="s">
         <v>14</v>
       </c>
@@ -5734,7 +5718,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="76" t="s">
         <v>41</v>
       </c>
@@ -5761,7 +5745,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="76" t="s">
         <v>330</v>
       </c>
@@ -5788,7 +5772,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="76" t="s">
         <v>58</v>
       </c>
@@ -5824,479 +5808,144 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:E35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="36.44140625" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F546759E-1E7A-4FBA-BCE7-8747DD03CB19}">
+  <dimension ref="B2:E12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>335</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>336</v>
+        <v>193</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>377</v>
       </c>
       <c r="E2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>338</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>339</v>
+        <v>191</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>377</v>
       </c>
       <c r="E3" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C4" t="s">
-        <v>339</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>378</v>
       </c>
       <c r="E4" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>338</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>339</v>
+        <v>195</v>
       </c>
       <c r="D5" t="s">
-        <v>5</v>
+        <v>379</v>
       </c>
       <c r="E5" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>338</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>339</v>
+        <v>209</v>
       </c>
       <c r="D6" t="s">
-        <v>5</v>
+        <v>380</v>
       </c>
       <c r="E6" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>338</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>339</v>
+        <v>181</v>
       </c>
       <c r="D7" t="s">
-        <v>5</v>
+        <v>381</v>
       </c>
       <c r="E7" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>338</v>
-      </c>
-      <c r="C8" t="s">
-        <v>339</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>5</v>
+        <v>382</v>
       </c>
       <c r="E8" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>338</v>
-      </c>
-      <c r="C9" t="s">
-        <v>346</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
+        <v>383</v>
+      </c>
+      <c r="E9" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>384</v>
+      </c>
+      <c r="E10" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>330</v>
+      </c>
+      <c r="D11" t="s">
+        <v>386</v>
+      </c>
+      <c r="E11" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>58</v>
       </c>
-      <c r="E9" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>338</v>
-      </c>
-      <c r="C10" t="s">
-        <v>346</v>
-      </c>
-      <c r="D10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>338</v>
-      </c>
-      <c r="C11" t="s">
-        <v>346</v>
-      </c>
-      <c r="D11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
-        <v>338</v>
-      </c>
-      <c r="C12" t="s">
-        <v>339</v>
-      </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>385</v>
       </c>
       <c r="E12" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
-        <v>338</v>
-      </c>
-      <c r="C13" t="s">
-        <v>339</v>
-      </c>
-      <c r="D13" t="s">
-        <v>351</v>
-      </c>
-      <c r="E13" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>338</v>
-      </c>
-      <c r="C14" t="s">
-        <v>346</v>
-      </c>
-      <c r="D14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
-        <v>338</v>
-      </c>
-      <c r="C15" t="s">
-        <v>353</v>
-      </c>
-      <c r="D15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
-        <v>338</v>
-      </c>
-      <c r="C16" t="s">
-        <v>353</v>
-      </c>
-      <c r="D16" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
-        <v>338</v>
-      </c>
-      <c r="C17" t="s">
-        <v>353</v>
-      </c>
-      <c r="D17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
-        <v>338</v>
-      </c>
-      <c r="C18" t="s">
-        <v>357</v>
-      </c>
-      <c r="D18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C19" t="s">
-        <v>339</v>
-      </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C20" t="s">
-        <v>339</v>
-      </c>
-      <c r="D20" t="s">
-        <v>351</v>
-      </c>
-      <c r="E20" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C21" t="s">
-        <v>339</v>
-      </c>
-      <c r="D21" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C22" t="s">
-        <v>339</v>
-      </c>
-      <c r="D22" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C23" t="s">
-        <v>339</v>
-      </c>
-      <c r="D23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C24" t="s">
-        <v>339</v>
-      </c>
-      <c r="D24" t="s">
-        <v>41</v>
-      </c>
-      <c r="E24" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="13">
-        <v>46092</v>
-      </c>
-      <c r="C25" t="s">
-        <v>339</v>
-      </c>
-      <c r="D25" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="13">
-        <v>46119</v>
-      </c>
-      <c r="C26" t="s">
-        <v>346</v>
-      </c>
-      <c r="E26" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="13">
-        <v>46119</v>
-      </c>
-      <c r="C27" t="s">
-        <v>346</v>
-      </c>
-      <c r="D27" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B28" s="13">
-        <v>46119</v>
-      </c>
-      <c r="C28" t="s">
-        <v>346</v>
-      </c>
-      <c r="D28" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B29" s="13">
-        <v>46119</v>
-      </c>
-      <c r="C29" t="s">
-        <v>346</v>
-      </c>
-      <c r="D29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B30" s="13">
-        <v>46121</v>
-      </c>
-      <c r="C30" t="s">
-        <v>365</v>
-      </c>
-      <c r="D30" t="s">
-        <v>366</v>
-      </c>
-      <c r="E30" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B31" s="13">
-        <v>46121</v>
-      </c>
-      <c r="C31" t="s">
-        <v>368</v>
-      </c>
-      <c r="D31" t="s">
-        <v>369</v>
-      </c>
-      <c r="E31" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B32" s="13">
-        <v>46126</v>
-      </c>
-      <c r="C32" t="s">
-        <v>371</v>
-      </c>
-      <c r="D32" t="s">
-        <v>372</v>
-      </c>
-      <c r="E32" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B33" s="13">
-        <v>46134</v>
-      </c>
-      <c r="C33" t="s">
-        <v>374</v>
-      </c>
-      <c r="E33" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B34" s="13">
-        <v>46134</v>
-      </c>
-      <c r="C34" t="s">
-        <v>339</v>
-      </c>
-      <c r="E34" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B35" s="13">
-        <v>46160</v>
-      </c>
-      <c r="C35" t="s">
-        <v>346</v>
-      </c>
-      <c r="E35" t="s">
-        <v>416</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -6305,147 +5954,491 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F546759E-1E7A-4FBA-BCE7-8747DD03CB19}">
-  <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="B2:E35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D2" t="s">
-        <v>377</v>
-      </c>
-      <c r="E2" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+      <c r="E3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>338</v>
+      </c>
+      <c r="C4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>191</v>
-      </c>
-      <c r="D3" t="s">
-        <v>377</v>
-      </c>
-      <c r="E3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+      <c r="E4" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C5" t="s">
+        <v>339</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>338</v>
+      </c>
+      <c r="C7" t="s">
+        <v>339</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>338</v>
+      </c>
+      <c r="C8" t="s">
+        <v>339</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C9" t="s">
+        <v>346</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>338</v>
+      </c>
+      <c r="C10" t="s">
+        <v>346</v>
+      </c>
+      <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11" t="s">
+        <v>346</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>338</v>
+      </c>
+      <c r="C12" t="s">
+        <v>339</v>
+      </c>
+      <c r="D12" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
-        <v>378</v>
-      </c>
-      <c r="E4" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
+      <c r="E12" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>338</v>
+      </c>
+      <c r="C13" t="s">
+        <v>339</v>
+      </c>
+      <c r="D13" t="s">
+        <v>351</v>
+      </c>
+      <c r="E13" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>338</v>
+      </c>
+      <c r="C14" t="s">
+        <v>346</v>
+      </c>
+      <c r="D14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>338</v>
+      </c>
+      <c r="C15" t="s">
+        <v>353</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>338</v>
+      </c>
+      <c r="C16" t="s">
+        <v>353</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>338</v>
+      </c>
+      <c r="C17" t="s">
+        <v>353</v>
+      </c>
+      <c r="D17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>338</v>
+      </c>
+      <c r="C18" t="s">
+        <v>357</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C19" t="s">
+        <v>339</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C20" t="s">
+        <v>339</v>
+      </c>
+      <c r="D20" t="s">
+        <v>351</v>
+      </c>
+      <c r="E20" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C21" t="s">
+        <v>339</v>
+      </c>
+      <c r="D21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C22" t="s">
+        <v>339</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C23" t="s">
+        <v>339</v>
+      </c>
+      <c r="D23" t="s">
         <v>20</v>
       </c>
-      <c r="C5" t="s">
-        <v>195</v>
-      </c>
-      <c r="D5" t="s">
-        <v>379</v>
-      </c>
-      <c r="E5" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D6" t="s">
-        <v>380</v>
-      </c>
-      <c r="E6" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="E23" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C24" t="s">
+        <v>339</v>
+      </c>
+      <c r="D24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="13">
+        <v>46092</v>
+      </c>
+      <c r="C25" t="s">
+        <v>339</v>
+      </c>
+      <c r="D25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="13">
+        <v>46119</v>
+      </c>
+      <c r="C26" t="s">
+        <v>346</v>
+      </c>
+      <c r="E26" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="13">
+        <v>46119</v>
+      </c>
+      <c r="C27" t="s">
+        <v>346</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="13">
+        <v>46119</v>
+      </c>
+      <c r="C28" t="s">
+        <v>346</v>
+      </c>
+      <c r="D28" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D7" t="s">
-        <v>381</v>
-      </c>
-      <c r="E7" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="E28" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="13">
+        <v>46119</v>
+      </c>
+      <c r="C29" t="s">
+        <v>346</v>
+      </c>
+      <c r="D29" t="s">
         <v>22</v>
       </c>
-      <c r="D8" t="s">
-        <v>382</v>
-      </c>
-      <c r="E8" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" t="s">
-        <v>383</v>
-      </c>
-      <c r="E9" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>384</v>
-      </c>
-      <c r="E10" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>330</v>
-      </c>
-      <c r="D11" t="s">
-        <v>386</v>
-      </c>
-      <c r="E11" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" t="s">
-        <v>385</v>
-      </c>
-      <c r="E12" t="s">
-        <v>398</v>
+      <c r="E29" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="13">
+        <v>46121</v>
+      </c>
+      <c r="C30" t="s">
+        <v>365</v>
+      </c>
+      <c r="D30" t="s">
+        <v>366</v>
+      </c>
+      <c r="E30" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="13">
+        <v>46121</v>
+      </c>
+      <c r="C31" t="s">
+        <v>368</v>
+      </c>
+      <c r="D31" t="s">
+        <v>369</v>
+      </c>
+      <c r="E31" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="13">
+        <v>46126</v>
+      </c>
+      <c r="C32" t="s">
+        <v>371</v>
+      </c>
+      <c r="D32" t="s">
+        <v>372</v>
+      </c>
+      <c r="E32" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="13">
+        <v>46134</v>
+      </c>
+      <c r="C33" t="s">
+        <v>374</v>
+      </c>
+      <c r="E33" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="13">
+        <v>46134</v>
+      </c>
+      <c r="C34" t="s">
+        <v>339</v>
+      </c>
+      <c r="E34" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="13">
+        <v>46160</v>
+      </c>
+      <c r="C35" t="s">
+        <v>346</v>
+      </c>
+      <c r="E35" t="s">
+        <v>416</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5264800B-FF6A-4F22-B8F4-02E853F50533}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6462,15 +6455,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090862990C7B69B4FACED7B33CDEA6B2D" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cb2feda0469996778cb97eaa0df7bf34">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ddaf961-75a3-44f9-b9a0-6c4032ed836e" xmlns:ns3="6eb7e908-d61c-4846-9ec9-1ad75cf16705" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ee5c23c3434d1001a3ba2f51c828df17" ns2:_="" ns3:_="">
     <xsd:import namespace="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
@@ -6711,6 +6695,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
   <ds:schemaRefs>
@@ -6723,14 +6716,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{186B4DCA-A60A-452A-99AD-03FF95333E10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6749,6 +6734,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" enabled="0" method="" siteId="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" removed="1"/>

</xml_diff>

<commit_message>
revert to original csv name
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50726C49-A423-423D-AC6D-B4556D156766}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D8BF000-30E9-402D-B9A2-F31D94FEDF31}"/>
   <bookViews>
-    <workbookView xWindow="7920" yWindow="1320" windowWidth="19275" windowHeight="13800" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="documentos" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="438">
   <si>
     <t>Documentos por Operación — Torre de Control CCR</t>
   </si>
@@ -1408,6 +1408,12 @@
   </si>
   <si>
     <t xml:space="preserve">Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa. </t>
+  </si>
+  <si>
+    <t>clausulas</t>
+  </si>
+  <si>
+    <t>generacion automática de filtros con base en csv generado por el dashboard de clausulas del banco</t>
   </si>
 </sst>
 </file>
@@ -2175,16 +2181,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
@@ -2532,12 +2538,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
     </row>
     <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5218,7 +5224,7 @@
       <c r="E34" s="18" t="s">
         <v>281</v>
       </c>
-      <c r="F34" s="86" t="s">
+      <c r="F34" s="88" t="s">
         <v>282</v>
       </c>
       <c r="G34" s="21" t="s">
@@ -5238,7 +5244,7 @@
       <c r="E35" s="23" t="s">
         <v>285</v>
       </c>
-      <c r="F35" s="87"/>
+      <c r="F35" s="89"/>
       <c r="G35" s="25" t="s">
         <v>286</v>
       </c>
@@ -5256,7 +5262,7 @@
       <c r="E36" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="F36" s="87"/>
+      <c r="F36" s="89"/>
       <c r="G36" s="25" t="s">
         <v>286</v>
       </c>
@@ -5955,7 +5961,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:E35"/>
+  <dimension ref="B2:E36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -6427,6 +6433,17 @@
       </c>
       <c r="E35" t="s">
         <v>416</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="13">
+        <v>46169</v>
+      </c>
+      <c r="C36" t="s">
+        <v>436</v>
+      </c>
+      <c r="E36" t="s">
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -6444,17 +6461,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6eb7e908-d61c-4846-9ec9-1ad75cf16705" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ddaf961-75a3-44f9-b9a0-6c4032ed836e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090862990C7B69B4FACED7B33CDEA6B2D" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cb2feda0469996778cb97eaa0df7bf34">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ddaf961-75a3-44f9-b9a0-6c4032ed836e" xmlns:ns3="6eb7e908-d61c-4846-9ec9-1ad75cf16705" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ee5c23c3434d1001a3ba2f51c828df17" ns2:_="" ns3:_="">
     <xsd:import namespace="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
@@ -6695,6 +6701,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6eb7e908-d61c-4846-9ec9-1ad75cf16705" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ddaf961-75a3-44f9-b9a0-6c4032ed836e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -6705,17 +6722,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6eb7e908-d61c-4846-9ec9-1ad75cf16705"/>
-    <ds:schemaRef ds:uri="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{186B4DCA-A60A-452A-99AD-03FF95333E10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6734,6 +6740,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6eb7e908-d61c-4846-9ec9-1ad75cf16705"/>
+    <ds:schemaRef ds:uri="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
correccion tabla clausulas + 180
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D8BF000-30E9-402D-B9A2-F31D94FEDF31}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B6F238B-AEDD-495E-9E3D-FB3AAEC7FE9B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="documentos" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'clausulas 180 dias'!$B$4:$K$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">documentos!$A$3:$D$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">documentos!$A$3:$D$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'productos criticos'!$B$3:$G$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="441">
   <si>
     <t>Documentos por Operación — Torre de Control CCR</t>
   </si>
@@ -1415,6 +1415,15 @@
   <si>
     <t>generacion automática de filtros con base en csv generado por el dashboard de clausulas del banco</t>
   </si>
+  <si>
+    <t>https://idbg.sharepoint.com/teams/ez-CR-L1157/_layouts/15/DocIdRedir.aspx?ID=EZIDB0003356-828744887-9</t>
+  </si>
+  <si>
+    <t>EZIDB0003356-828744887-9</t>
+  </si>
+  <si>
+    <t>https://idbg.sharepoint.com/teams/EZ-CR-LON/CR-L1065/_layouts/15/DocIdRedir.aspx?ID=EZIDB0000195-998400382-110</t>
+  </si>
 </sst>
 </file>
 
@@ -1423,7 +1432,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-10409]dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1566,11 +1575,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <u/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -1932,7 +1936,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2128,9 +2132,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2527,7 +2528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="66" customWidth="1"/>
@@ -2538,12 +2539,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
     </row>
     <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2570,7 +2571,7 @@
       <c r="C4" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="68" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2584,7 +2585,7 @@
       <c r="C5" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="68" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2598,7 +2599,7 @@
       <c r="C6" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="69" t="s">
+      <c r="D6" s="68" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2612,7 +2613,7 @@
       <c r="C7" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="69" t="s">
+      <c r="D7" s="68" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2626,7 +2627,7 @@
       <c r="C8" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="68" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2640,7 +2641,7 @@
       <c r="C9" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="69" t="s">
+      <c r="D9" s="68" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2654,7 +2655,7 @@
       <c r="C10" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="69" t="s">
+      <c r="D10" s="68" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2668,7 +2669,7 @@
       <c r="C11" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="69" t="s">
+      <c r="D11" s="68" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2682,7 +2683,7 @@
       <c r="C12" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="69" t="s">
+      <c r="D12" s="68" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2696,7 +2697,7 @@
       <c r="C13" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="69" t="s">
+      <c r="D13" s="68" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2710,7 +2711,7 @@
       <c r="C14" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="69" t="s">
+      <c r="D14" s="68" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2724,7 +2725,7 @@
       <c r="C15" s="68" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="69" t="s">
+      <c r="D15" s="68" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2738,7 +2739,7 @@
       <c r="C16" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="69" t="s">
+      <c r="D16" s="68" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2752,7 +2753,7 @@
       <c r="C17" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="69" t="s">
+      <c r="D17" s="68" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2778,7 +2779,7 @@
       <c r="C19" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="69" t="s">
+      <c r="D19" s="68" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2792,7 +2793,7 @@
       <c r="C20" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="69" t="s">
+      <c r="D20" s="68" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2806,7 +2807,7 @@
       <c r="C21" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="69" t="s">
+      <c r="D21" s="68" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2820,7 +2821,7 @@
       <c r="C22" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="69" t="s">
+      <c r="D22" s="68" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2834,7 +2835,7 @@
       <c r="C23" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="69" t="s">
+      <c r="D23" s="68" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2848,7 +2849,7 @@
       <c r="C24" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="69" t="s">
+      <c r="D24" s="68" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2862,7 +2863,7 @@
       <c r="C25" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="D25" s="69" t="s">
+      <c r="D25" s="68" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2876,7 +2877,7 @@
       <c r="C26" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="69" t="s">
+      <c r="D26" s="68" t="s">
         <v>60</v>
       </c>
     </row>
@@ -2890,7 +2891,7 @@
       <c r="C27" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="69" t="s">
+      <c r="D27" s="68" t="s">
         <v>63</v>
       </c>
     </row>
@@ -2904,7 +2905,7 @@
       <c r="C28" s="68" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="69" t="s">
+      <c r="D28" s="68" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2918,7 +2919,7 @@
       <c r="C29" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="D29" s="69" t="s">
+      <c r="D29" s="68" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2932,7 +2933,7 @@
       <c r="C30" s="68" t="s">
         <v>66</v>
       </c>
-      <c r="D30" s="69" t="s">
+      <c r="D30" s="68" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2946,7 +2947,7 @@
       <c r="C31" s="68" t="s">
         <v>68</v>
       </c>
-      <c r="D31" s="69" t="s">
+      <c r="D31" s="68" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2960,7 +2961,7 @@
       <c r="C32" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="D32" s="69" t="s">
+      <c r="D32" s="68" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2974,7 +2975,7 @@
       <c r="C33" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="D33" s="69" t="s">
+      <c r="D33" s="68" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2988,7 +2989,7 @@
       <c r="C34" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="D34" s="69" t="s">
+      <c r="D34" s="68" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3002,7 +3003,7 @@
       <c r="C35" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="D35" s="69" t="s">
+      <c r="D35" s="68" t="s">
         <v>78</v>
       </c>
     </row>
@@ -3016,7 +3017,7 @@
       <c r="C36" s="68" t="s">
         <v>79</v>
       </c>
-      <c r="D36" s="69" t="s">
+      <c r="D36" s="68" t="s">
         <v>80</v>
       </c>
     </row>
@@ -3030,7 +3031,7 @@
       <c r="C37" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="D37" s="69" t="s">
+      <c r="D37" s="68" t="s">
         <v>82</v>
       </c>
     </row>
@@ -3044,7 +3045,7 @@
       <c r="C38" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="D38" s="69" t="s">
+      <c r="D38" s="68" t="s">
         <v>84</v>
       </c>
     </row>
@@ -3058,7 +3059,7 @@
       <c r="C39" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="69" t="s">
+      <c r="D39" s="68" t="s">
         <v>86</v>
       </c>
     </row>
@@ -3072,7 +3073,7 @@
       <c r="C40" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="69" t="s">
+      <c r="D40" s="68" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3086,7 +3087,7 @@
       <c r="C41" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="D41" s="69" t="s">
+      <c r="D41" s="68" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3100,7 +3101,7 @@
       <c r="C42" s="68" t="s">
         <v>91</v>
       </c>
-      <c r="D42" s="69" t="s">
+      <c r="D42" s="68" t="s">
         <v>92</v>
       </c>
     </row>
@@ -3114,7 +3115,7 @@
       <c r="C43" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="D43" s="69" t="s">
+      <c r="D43" s="68" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3128,7 +3129,7 @@
       <c r="C44" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="D44" s="69" t="s">
+      <c r="D44" s="68" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3142,7 +3143,7 @@
       <c r="C45" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="D45" s="69" t="s">
+      <c r="D45" s="68" t="s">
         <v>99</v>
       </c>
     </row>
@@ -3156,7 +3157,7 @@
       <c r="C46" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="D46" s="69" t="s">
+      <c r="D46" s="68" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3170,7 +3171,7 @@
       <c r="C47" s="68" t="s">
         <v>103</v>
       </c>
-      <c r="D47" s="69" t="s">
+      <c r="D47" s="68" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3184,7 +3185,7 @@
       <c r="C48" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="D48" s="69" t="s">
+      <c r="D48" s="68" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3198,7 +3199,7 @@
       <c r="C49" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="D49" s="69" t="s">
+      <c r="D49" s="68" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3212,7 +3213,7 @@
       <c r="C50" s="68" t="s">
         <v>110</v>
       </c>
-      <c r="D50" s="69" t="s">
+      <c r="D50" s="68" t="s">
         <v>111</v>
       </c>
     </row>
@@ -3226,7 +3227,7 @@
       <c r="C51" s="68" t="s">
         <v>112</v>
       </c>
-      <c r="D51" s="69" t="s">
+      <c r="D51" s="68" t="s">
         <v>113</v>
       </c>
     </row>
@@ -3240,7 +3241,7 @@
       <c r="C52" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="D52" s="69" t="s">
+      <c r="D52" s="68" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3254,7 +3255,7 @@
       <c r="C53" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="D53" s="69" t="s">
+      <c r="D53" s="68" t="s">
         <v>117</v>
       </c>
     </row>
@@ -3268,7 +3269,7 @@
       <c r="C54" s="68" t="s">
         <v>118</v>
       </c>
-      <c r="D54" s="69" t="s">
+      <c r="D54" s="68" t="s">
         <v>119</v>
       </c>
     </row>
@@ -3282,7 +3283,7 @@
       <c r="C55" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="D55" s="69" t="s">
+      <c r="D55" s="68" t="s">
         <v>122</v>
       </c>
     </row>
@@ -3296,7 +3297,9 @@
       <c r="C56" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="D56" s="68"/>
+      <c r="D56" s="68" t="s">
+        <v>440</v>
+      </c>
     </row>
     <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="67" t="s">
@@ -3308,7 +3311,7 @@
       <c r="C57" s="68" t="s">
         <v>124</v>
       </c>
-      <c r="D57" s="69" t="s">
+      <c r="D57" s="68" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3322,24 +3325,40 @@
       <c r="C58" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="D58" s="69" t="s">
+      <c r="D58" s="68" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="67" t="s">
+        <v>58</v>
+      </c>
+      <c r="B59" s="68" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="68" t="s">
+        <v>439</v>
+      </c>
+      <c r="D59" s="68" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="B59" s="68" t="s">
+      <c r="B60" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="C59" s="68" t="s">
+      <c r="C60" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="D59" s="68"/>
+      <c r="D60" s="68" t="s">
+        <v>122</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D59" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:D60" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -4210,7 +4229,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4304,7 +4323,7 @@
       </c>
       <c r="K5" s="10">
         <f t="shared" ref="K5:K13" ca="1" si="0">J5-TODAY()</f>
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -4337,7 +4356,7 @@
       </c>
       <c r="K6" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -4370,7 +4389,7 @@
       </c>
       <c r="K7" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -4403,7 +4422,7 @@
       </c>
       <c r="K8" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -4436,7 +4455,7 @@
       </c>
       <c r="K9" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -4469,7 +4488,7 @@
       </c>
       <c r="K10" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="2:11" ht="24" x14ac:dyDescent="0.25">
@@ -4502,7 +4521,7 @@
       </c>
       <c r="K11" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -4535,7 +4554,7 @@
       </c>
       <c r="K12" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -4568,7 +4587,7 @@
       </c>
       <c r="K13" s="10">
         <f t="shared" ca="1" si="0"/>
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="2:11" ht="24" x14ac:dyDescent="0.25">
@@ -4601,7 +4620,7 @@
       </c>
       <c r="K14" s="10">
         <f t="shared" ref="K14:K15" ca="1" si="1">J14-TODAY()</f>
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -4634,7 +4653,7 @@
       </c>
       <c r="K15" s="10">
         <f t="shared" ca="1" si="1"/>
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -4643,7 +4662,7 @@
       <sortCondition ref="K4:K13"/>
     </sortState>
   </autoFilter>
-  <phoneticPr fontId="23" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5013,7 +5032,7 @@
       <c r="G21" s="23"/>
     </row>
     <row r="22" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="77" t="s">
+      <c r="B22" s="76" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="30" t="s">
@@ -5026,10 +5045,10 @@
         <v>264</v>
       </c>
       <c r="F22" s="30"/>
-      <c r="G22" s="78"/>
+      <c r="G22" s="77"/>
     </row>
     <row r="23" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="79" t="s">
+      <c r="B23" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -5039,10 +5058,10 @@
         <v>225</v>
       </c>
       <c r="E23" s="23"/>
-      <c r="G23" s="80"/>
+      <c r="G23" s="79"/>
     </row>
     <row r="24" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="79" t="s">
+      <c r="B24" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -5052,10 +5071,10 @@
         <v>225</v>
       </c>
       <c r="E24" s="23"/>
-      <c r="G24" s="80"/>
+      <c r="G24" s="79"/>
     </row>
     <row r="25" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="79" t="s">
+      <c r="B25" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -5065,10 +5084,10 @@
         <v>225</v>
       </c>
       <c r="E25" s="23"/>
-      <c r="G25" s="80"/>
+      <c r="G25" s="79"/>
     </row>
     <row r="26" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="79" t="s">
+      <c r="B26" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -5078,10 +5097,10 @@
         <v>225</v>
       </c>
       <c r="E26" s="23"/>
-      <c r="G26" s="80"/>
+      <c r="G26" s="79"/>
     </row>
     <row r="27" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="79" t="s">
+      <c r="B27" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -5091,10 +5110,10 @@
         <v>225</v>
       </c>
       <c r="E27" s="23"/>
-      <c r="G27" s="80"/>
+      <c r="G27" s="79"/>
     </row>
     <row r="28" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="79" t="s">
+      <c r="B28" s="78" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -5109,25 +5128,25 @@
       <c r="F28" s="23" t="s">
         <v>427</v>
       </c>
-      <c r="G28" s="80"/>
+      <c r="G28" s="79"/>
     </row>
     <row r="29" spans="2:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="82" t="s">
+      <c r="C29" s="81" t="s">
         <v>417</v>
       </c>
-      <c r="D29" s="83" t="s">
+      <c r="D29" s="82" t="s">
         <v>228</v>
       </c>
-      <c r="E29" s="84" t="s">
+      <c r="E29" s="83" t="s">
         <v>418</v>
       </c>
       <c r="F29" s="23" t="s">
         <v>427</v>
       </c>
-      <c r="G29" s="85" t="s">
+      <c r="G29" s="84" t="s">
         <v>265</v>
       </c>
     </row>
@@ -5224,7 +5243,7 @@
       <c r="E34" s="18" t="s">
         <v>281</v>
       </c>
-      <c r="F34" s="88" t="s">
+      <c r="F34" s="87" t="s">
         <v>282</v>
       </c>
       <c r="G34" s="21" t="s">
@@ -5244,7 +5263,7 @@
       <c r="E35" s="23" t="s">
         <v>285</v>
       </c>
-      <c r="F35" s="89"/>
+      <c r="F35" s="88"/>
       <c r="G35" s="25" t="s">
         <v>286</v>
       </c>
@@ -5262,7 +5281,7 @@
       <c r="E36" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="F36" s="89"/>
+      <c r="F36" s="88"/>
       <c r="G36" s="25" t="s">
         <v>286</v>
       </c>
@@ -5397,13 +5416,13 @@
       <c r="C2" s="65"/>
     </row>
     <row r="4" spans="2:17" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="75" t="s">
+      <c r="B4" s="74" t="s">
         <v>174</v>
       </c>
-      <c r="C4" s="75" t="s">
+      <c r="C4" s="74" t="s">
         <v>399</v>
       </c>
-      <c r="D4" s="74" t="s">
+      <c r="D4" s="73" t="s">
         <v>387</v>
       </c>
       <c r="E4" s="63" t="s">
@@ -5438,13 +5457,13 @@
       </c>
     </row>
     <row r="5" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="76" t="s">
+      <c r="B5" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="76" t="s">
+      <c r="C5" s="75" t="s">
         <v>389</v>
       </c>
-      <c r="D5" s="70" t="s">
+      <c r="D5" s="69" t="s">
         <v>313</v>
       </c>
       <c r="E5" s="46" t="s">
@@ -5479,13 +5498,13 @@
       </c>
     </row>
     <row r="6" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="76" t="s">
+      <c r="B6" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="76" t="s">
+      <c r="C6" s="75" t="s">
         <v>390</v>
       </c>
-      <c r="D6" s="71" t="s">
+      <c r="D6" s="70" t="s">
         <v>317</v>
       </c>
       <c r="E6" s="48" t="s">
@@ -5520,13 +5539,13 @@
       </c>
     </row>
     <row r="7" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="76" t="s">
+      <c r="B7" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="76" t="s">
+      <c r="C7" s="75" t="s">
         <v>391</v>
       </c>
-      <c r="D7" s="71" t="s">
+      <c r="D7" s="70" t="s">
         <v>317</v>
       </c>
       <c r="E7" s="48" t="s">
@@ -5561,13 +5580,13 @@
       </c>
     </row>
     <row r="8" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="76" t="s">
+      <c r="B8" s="75" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="76" t="s">
+      <c r="C8" s="75" t="s">
         <v>392</v>
       </c>
-      <c r="D8" s="71" t="s">
+      <c r="D8" s="70" t="s">
         <v>317</v>
       </c>
       <c r="E8" s="48" t="s">
@@ -5602,13 +5621,13 @@
       </c>
     </row>
     <row r="9" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="76" t="s">
+      <c r="B9" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="76" t="s">
+      <c r="C9" s="75" t="s">
         <v>393</v>
       </c>
-      <c r="D9" s="70" t="s">
+      <c r="D9" s="69" t="s">
         <v>313</v>
       </c>
       <c r="E9" s="48" t="s">
@@ -5643,13 +5662,13 @@
       </c>
     </row>
     <row r="10" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="76" t="s">
+      <c r="C10" s="75" t="s">
         <v>394</v>
       </c>
-      <c r="D10" s="72" t="s">
+      <c r="D10" s="71" t="s">
         <v>325</v>
       </c>
       <c r="E10" s="58" t="s">
@@ -5684,13 +5703,13 @@
       </c>
     </row>
     <row r="11" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="76" t="s">
+      <c r="C11" s="75" t="s">
         <v>395</v>
       </c>
-      <c r="D11" s="71" t="s">
+      <c r="D11" s="70" t="s">
         <v>317</v>
       </c>
       <c r="E11" s="48" t="s">
@@ -5725,13 +5744,13 @@
       </c>
     </row>
     <row r="12" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="76" t="s">
+      <c r="B12" s="75" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="76" t="s">
+      <c r="C12" s="75" t="s">
         <v>396</v>
       </c>
-      <c r="D12" s="70" t="s">
+      <c r="D12" s="69" t="s">
         <v>313</v>
       </c>
       <c r="E12" s="48" t="s">
@@ -5752,13 +5771,13 @@
       </c>
     </row>
     <row r="13" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="75" t="s">
         <v>330</v>
       </c>
-      <c r="C13" s="76" t="s">
+      <c r="C13" s="75" t="s">
         <v>397</v>
       </c>
-      <c r="D13" s="73" t="s">
+      <c r="D13" s="72" t="s">
         <v>331</v>
       </c>
       <c r="E13" s="61" t="s">
@@ -5779,13 +5798,13 @@
       </c>
     </row>
     <row r="14" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="76" t="s">
+      <c r="C14" s="75" t="s">
         <v>398</v>
       </c>
-      <c r="D14" s="71" t="s">
+      <c r="D14" s="70" t="s">
         <v>317</v>
       </c>
       <c r="E14" s="48" t="s">
@@ -6702,6 +6721,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="6eb7e908-d61c-4846-9ec9-1ad75cf16705" xsi:nil="true"/>
@@ -6710,15 +6738,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6741,6 +6760,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -6751,14 +6778,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" enabled="0" method="" siteId="{9dfb1a05-5f1d-449a-8960-62abcb479e7d}" removed="1"/>

</xml_diff>

<commit_message>
actualiza codigo de colores de indicadores pmr
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1B3A4FF-E0D4-40F2-A73D-2B8281469A2E}"/>
+  <xr:revisionPtr revIDLastSave="143" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF2EAB07-5D96-4F5F-BD3B-B91100B57C3D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="400">
   <si>
     <t>Documentos por Operación — Torre de Control CCR</t>
   </si>
@@ -1290,6 +1290,12 @@
   </si>
   <si>
     <t>Asigna como analista 1 al responsible del equipo de operaciones</t>
+  </si>
+  <si>
+    <t>pmr</t>
+  </si>
+  <si>
+    <t>actualiza codigo de colores para indicadores tecnicos segun guía de pmr</t>
   </si>
 </sst>
 </file>
@@ -4980,7 +4986,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:E42"/>
+  <dimension ref="B2:E43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -5534,12 +5540,34 @@
         <v>397</v>
       </c>
     </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43" s="8">
+        <v>46171</v>
+      </c>
+      <c r="C43" t="s">
+        <v>398</v>
+      </c>
+      <c r="E43" t="s">
+        <v>399</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6eb7e908-d61c-4846-9ec9-1ad75cf16705" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ddaf961-75a3-44f9-b9a0-6c4032ed836e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090862990C7B69B4FACED7B33CDEA6B2D" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cb2feda0469996778cb97eaa0df7bf34">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ddaf961-75a3-44f9-b9a0-6c4032ed836e" xmlns:ns3="6eb7e908-d61c-4846-9ec9-1ad75cf16705" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ee5c23c3434d1001a3ba2f51c828df17" ns2:_="" ns3:_="">
     <xsd:import namespace="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
@@ -5780,17 +5808,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6eb7e908-d61c-4846-9ec9-1ad75cf16705" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ddaf961-75a3-44f9-b9a0-6c4032ed836e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5801,6 +5818,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6eb7e908-d61c-4846-9ec9-1ad75cf16705"/>
+    <ds:schemaRef ds:uri="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{186B4DCA-A60A-452A-99AD-03FF95333E10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5819,17 +5847,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A1C5BB8-2969-4B26-83EB-3E0EFA4C2B46}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6eb7e908-d61c-4846-9ec9-1ad75cf16705"/>
-    <ds:schemaRef ds:uri="4ddaf961-75a3-44f9-b9a0-6c4032ed836e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F155E963-344D-4195-BD2C-0A3B31EF9B00}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
actualizacion datos en excel
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF2EAB07-5D96-4F5F-BD3B-B91100B57C3D}"/>
+  <xr:revisionPtr revIDLastSave="168" documentId="13_ncr:1_{75047D51-A796-4CC0-AB19-45877F10B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5842BA85-CDBD-43C5-AB54-11BB4B75D9F3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3705" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="documentos" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">documentos!$A$3:$D$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'productos criticos'!$B$3:$G$34</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="402">
   <si>
     <t>Documentos por Operación — Torre de Control CCR</t>
   </si>
@@ -416,6 +419,9 @@
     <t>EZIDB0000195-998400382-110</t>
   </si>
   <si>
+    <t>https://idbg.sharepoint.com/teams/EZ-CR-LON/CR-L1065/_layouts/15/DocIdRedir.aspx?ID=EZIDB0000195-998400382-110</t>
+  </si>
+  <si>
     <t>EZIDB0000195-822257051-222</t>
   </si>
   <si>
@@ -425,6 +431,12 @@
     <t>EZIDB0000195-1127813953-75</t>
   </si>
   <si>
+    <t>EZIDB0003356-828744887-9</t>
+  </si>
+  <si>
+    <t>https://idbg.sharepoint.com/teams/ez-CR-L1157/_layouts/15/DocIdRedir.aspx?ID=EZIDB0003356-828744887-9</t>
+  </si>
+  <si>
     <t>Fecha revision</t>
   </si>
   <si>
@@ -461,15 +473,15 @@
     <t>SAIZ, ANA MARIA</t>
   </si>
   <si>
+    <t>PARAISO PINTO FURTADO LUZES, MARTA</t>
+  </si>
+  <si>
+    <t>ALARCON, ARTURO</t>
+  </si>
+  <si>
     <t>BIEHL, MARIA LORETO</t>
   </si>
   <si>
-    <t>ALARCON, ARTURO</t>
-  </si>
-  <si>
-    <t>PARAISO PINTO FURTADO LUZES, MARTA</t>
-  </si>
-  <si>
     <t>Abogado</t>
   </si>
   <si>
@@ -503,55 +515,70 @@
     <t>Apoyo a la tarea fiduciaria</t>
   </si>
   <si>
+    <t>OVIEDO BENAVIDES, GUSTAVO ALONSO</t>
+  </si>
+  <si>
     <t>OVIEDO BENAVIDES GUSTAVO ALONSO</t>
   </si>
   <si>
     <t>Equipo de ESG</t>
   </si>
   <si>
+    <t>HERNANDEZ, GABRIEL ANTONIO</t>
+  </si>
+  <si>
+    <t>ARELLANO CASTILLO, RAUL</t>
+  </si>
+  <si>
+    <t>FARINACCIO, ALESSANDRO</t>
+  </si>
+  <si>
     <t>PASTOR PIMENTEL, SEABELL ANNETTE</t>
   </si>
   <si>
-    <t>ARELLANO CASTILLO, RAUL</t>
-  </si>
-  <si>
-    <t>HERNANDEZ, GABRIEL ANTONIO</t>
-  </si>
-  <si>
     <t>PORTA GARCIA, RAIMON</t>
   </si>
   <si>
     <t>Analista 1</t>
   </si>
   <si>
+    <t>VEGA GAMBOA, JORGE DANIEL</t>
+  </si>
+  <si>
+    <t>MORA VARGAS, GREIVIN GERARDO</t>
+  </si>
+  <si>
     <t>BUSTOS BRENES, JUAN CARLOS</t>
   </si>
   <si>
+    <t>YGLESIAS FISCHEL, SOFIA</t>
+  </si>
+  <si>
     <t>BORBON MUNOZ, ALVARO</t>
   </si>
   <si>
     <t>Analista 2</t>
   </si>
   <si>
-    <t>MORA VARGAS, GREIVIN GERARDO</t>
-  </si>
-  <si>
-    <t>YGLESIAS FISCHEL, SOFIA</t>
+    <t>QUIROS SOLANO, FERNANDO ANDRES</t>
+  </si>
+  <si>
+    <t>Analista 3</t>
+  </si>
+  <si>
+    <t>GONZALO RODRIGUEZ VALVERDE</t>
   </si>
   <si>
     <t>VIVIANA NUNEZ DE URQUIDI</t>
   </si>
   <si>
-    <t>Analista 3</t>
+    <t>Analista 4</t>
   </si>
   <si>
     <t>GUTIERRES WUERZIUS, LUCIANO</t>
   </si>
   <si>
-    <t>Analista 4</t>
-  </si>
-  <si>
-    <t>GONZALO RODRIGUEZ VALVERDE</t>
+    <t>ALVAREZ GONZALEZ, OSCAR ANDRES</t>
   </si>
   <si>
     <t>Analista 5</t>
@@ -560,24 +587,6 @@
     <t>Analista 6</t>
   </si>
   <si>
-    <t>Programa</t>
-  </si>
-  <si>
-    <t>4871/OC-CR</t>
-  </si>
-  <si>
-    <t>3072/CH-CR</t>
-  </si>
-  <si>
-    <t>3071/OC-CR</t>
-  </si>
-  <si>
-    <t>4864/OC-CR</t>
-  </si>
-  <si>
-    <t>5823/OC-CR</t>
-  </si>
-  <si>
     <t>Fecha de corte: 06 abril 2026</t>
   </si>
   <si>
@@ -617,36 +626,42 @@
     <t>Delegaciones diseñadas, construidas, equipadas y operando bajo el enfoque de policía comunitaria</t>
   </si>
   <si>
+    <t>DP Limón y El Roble</t>
+  </si>
+  <si>
+    <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
+  </si>
+  <si>
+    <t>Centro de Mando y Control Policial construido, equipado y en funcionamiento</t>
+  </si>
+  <si>
+    <t>D+C obra y adenda para suministro de equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa. </t>
+  </si>
+  <si>
+    <t>Estrategia de comunicación social de los CCP, diseñada e implementada</t>
+  </si>
+  <si>
+    <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
+  </si>
+  <si>
+    <t>Municipalidades y grupos de sociedad civil capacitados y en prevención de violencia</t>
+  </si>
+  <si>
+    <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
+  </si>
+  <si>
     <t>Retrasado</t>
   </si>
   <si>
-    <t>DP Limón y El Roble</t>
-  </si>
-  <si>
-    <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
-  </si>
-  <si>
-    <t>Centro de Mando y Control Policial construido, equipado y en funcionamiento</t>
-  </si>
-  <si>
-    <t>D+C obra y adenda para suministro de equipo</t>
-  </si>
-  <si>
-    <t>Estrategia de comunicación social de los CCP, diseñada e implementada</t>
-  </si>
-  <si>
-    <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
-  </si>
-  <si>
-    <t>Municipalidades y grupos de sociedad civil capacitados y en prevención de violencia</t>
-  </si>
-  <si>
-    <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
-  </si>
-  <si>
     <t>CCP Perez Zeledón, San José y Goicoechea</t>
   </si>
   <si>
+    <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Modelo de gestión y atención de los CCP homologado, fortalecido y en funcionamiento </t>
   </si>
   <si>
@@ -704,7 +719,13 @@
     <t xml:space="preserve">Tramo Central Sifón – Sucre </t>
   </si>
   <si>
-    <t>En análisis por FMP y TSP junto con el OE sobre iguiente estado del proceso: declaración de infructuoso o cancelación.</t>
+    <t>Pausado</t>
+  </si>
+  <si>
+    <t>Contratación para el diseño y construcción del Tramo Central de la Ruta Nacional no. 35</t>
+  </si>
+  <si>
+    <t>En análisis por FMP y TSP junto con el OE sobre siguiente estado del proceso: declaración de infructuoso, cancelación, o nueva fuente de financiamiento.</t>
   </si>
   <si>
     <t>1.1 Tiempo promedio de recorrido por vehículo en el tramo Florencia RN-1
@@ -713,11 +734,17 @@
 1.5. Sitios de la vía en el tramo de Abundancia Sifón (Tramo Central) afectados por inundaciones debido a precipitaciones con un período de retorno de 100 años.</t>
   </si>
   <si>
+    <t xml:space="preserve">Obras complementarias en el Tramo Central Sección Sucre – Abundancia </t>
+  </si>
+  <si>
     <t>Punta Sur de la RN-35 diseñado y construido</t>
   </si>
   <si>
+    <t xml:space="preserve">Contratación para el diseño y construcción de la Punta Sur de la Ruta Nacional no. 35 </t>
+  </si>
+  <si>
     <t>Lote 1 firmado
-Lote 2 en revisión jurídica del MOPT para firma de enmienda ya revisada y con NOB del Banco.</t>
+Lote 2 firmado.</t>
   </si>
   <si>
     <t>1.1 Tiempo promedio de recorrido por vehículo en el tramo Florencia RN-1
@@ -725,7 +752,46 @@
 1.3. Nivel de seguridad vial (cantidad de estrellas mediante la metodología de iRAP) de la RN-35</t>
   </si>
   <si>
+    <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
+  </si>
+  <si>
+    <t>Contratación de para el diseño y construcción de los sistemas de iluminación vial para la Punta Norte de la RN No. 35 (Sección ciudad Quesada / Florencia)</t>
+  </si>
+  <si>
+    <t>Número de funcionarios municipales capacitados</t>
+  </si>
+  <si>
     <t>Consultor individual que realice el PCR de operación</t>
+  </si>
+  <si>
+    <t>Número de cantones con Planes Viales Quinquenales de conservación y desarrollo elaborados</t>
+  </si>
+  <si>
+    <t>Manuales de seguridad vial y gestión socioambiental elaborados</t>
+  </si>
+  <si>
+    <t>Sistema de Gestión de activos viales implementado</t>
+  </si>
+  <si>
+    <t>Cantones con intervención de seguridad vial</t>
+  </si>
+  <si>
+    <t>Mantenimiento rutinario por estándares realizado a través de microempresas</t>
+  </si>
+  <si>
+    <t>Puentes construidos o rehabilitados</t>
+  </si>
+  <si>
+    <t>Construcción de puentes (paquetes), rehabilitados (Incluye diseño adaptados a cambio climático).</t>
+  </si>
+  <si>
+    <t>Evaluación Ex Post de resultados pendiente</t>
+  </si>
+  <si>
+    <t>Caminos cantonales rehabilitados</t>
+  </si>
+  <si>
+    <t>Rehabilitación de caminos (paquetes)</t>
   </si>
   <si>
     <t>1.1 Densidad de vías cantonales en buen estado
@@ -893,6 +959,18 @@
     <t>Ciclo I-2026 (Con corte de datos a dic 2025)</t>
   </si>
   <si>
+    <t>Programa</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Calificación Calculada</t>
+  </si>
+  <si>
+    <t>Calificación Validada</t>
+  </si>
+  <si>
     <t>Desembolsos</t>
   </si>
   <si>
@@ -920,6 +998,9 @@
     <t>Plan Acción 2026</t>
   </si>
   <si>
+    <t>Programa de Infraestructura de Transporte</t>
+  </si>
+  <si>
     <t>ALERTA</t>
   </si>
   <si>
@@ -932,30 +1013,45 @@
     <t>Asegurar la finalización de pagos de obras complementarias y expropiaciones, así como gastos de ruta 35 con cargo a la operación.</t>
   </si>
   <si>
+    <t>Programa Red Vial Cantonal II</t>
+  </si>
+  <si>
     <t>SATISFACTORIO</t>
   </si>
   <si>
     <t>No se advierten problemas para mantener la clasificación (operación en cierre)</t>
   </si>
   <si>
+    <t>Programa de Infraestructura Vial y promoción de Asociaciones Público-Privadas (APP)</t>
+  </si>
+  <si>
     <t>No se anticipa riesgo de cambio de clasificación en 2026. Para mantener el indicador de desembolsos en satisfactorio sólo necesita desembolsar $9m en 2026 ($21,6m planeados). Riesgo medio de que SPI y CPI pasen a alerta en función de los gastos realmente reportados para 2026, pero los desembolsos, SPI(a) y CPI(a) mantendrían la operación en satisfactorio.</t>
   </si>
   <si>
     <t>Asegurar un desembolso de al menos $9m en 2026. Monitorear avance financiero de intercambios y Taras la Lima para evaluar impacto de metas físicas y financieras en 2027.</t>
   </si>
   <si>
+    <t>Programa de Infraestructura Vial y Movilidad Urbana: conectividad resiliente</t>
+  </si>
+  <si>
     <t>El indicador de desembolsos requiere que se desmbolse el total planeado para 2026 ($20,2m) para mantenerse en alerta (requiere cerca de $35m para pasar a satisfactorio). El SPI probablemente pasará a alerta en 2026 y el SPI(a) requiere ejecutar alrededor de $8m en punta sur para mantenerse satisfactorio. Combinación de desembolsos y SPI en alerta + SPI(a), CPI y CPI(a) en satisfactorio mantendrían la operación en satisfactorio.</t>
   </si>
   <si>
     <t>Asegurar al menos la meta de desembolsos de la operación ($20,2m) y garantizar que gastos de punta sur + obras complementarias de punta norte superen los $8m (80% de lo planeado).</t>
   </si>
   <si>
+    <t>Programa de Seguridad Ciudadana y Prevención de Violencia</t>
+  </si>
+  <si>
     <t>El indicador de desembolsos se mantendrá en satisfactorio, aun sin desembolsos adicionales. Indicadores SPI(a) y CPI(a) dependen de la finalización de obras planeadas para el 2026. (la operación ya finalizó las obras requeridas para el año y superará las metas físicas, pero como el simulador de la operación tiene errores, es difícil determinar exactamente el impacto de superar las metas).</t>
   </si>
   <si>
     <t>Asegurar la finalización de al menos 4 delegaciones policiales y 1 centro cívico en 2026.</t>
   </si>
   <si>
+    <t>Programa Integral de Seguridad Ciudadana y Prevención de la Violencia para la Inclusión de Grupos Migrantes Vulnerables</t>
+  </si>
+  <si>
     <t>PROBLEMA</t>
   </si>
   <si>
@@ -965,6 +1061,12 @@
     <t>Monitorear e impulsar la ejecución de los procesos de regularización para alcanzar la meta de 60.000 procesos completados en 2026. Seguimiento al avance de CCP Upala y Unidad de Refugio.</t>
   </si>
   <si>
+    <t>Programa de Integración Fronteriza de Costa Rica</t>
+  </si>
+  <si>
+    <t>Mejora de la calidad del Sistema Educativo en Costa Rica</t>
+  </si>
+  <si>
     <t>Actualmente esperando ratificación. Considerando un proceso de firma de contrato inusual, se recomienda cambiar la clasificación a satisfactorio. El sistema seguirá clasificandolo como alerta automáticamente hasta que obtenga la ratificación.</t>
   </si>
   <si>
@@ -974,18 +1076,69 @@
     <t>CR-L1156</t>
   </si>
   <si>
+    <t>Apoyo al fortalecimiento y expansión del sistema nacional de cuidados de Costa Rica</t>
+  </si>
+  <si>
     <t>No indica</t>
   </si>
   <si>
     <t>Actualmente esperando ratificación. La operación no muestra clasificación ni gráfica de conteo de días hasta efectividad.</t>
   </si>
   <si>
+    <t>Segundo Programa de Energía Renovable, Transmisión y Distribución de Electricidad</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recién se firmó, por lo que para el próximo ciclo estarían contabilizando el plazo para alcanzar la elegibilidad. </t>
   </si>
   <si>
     <t>Monitorear proceso de elegibilidad.</t>
   </si>
   <si>
+    <t>3071/OC-CR</t>
+  </si>
+  <si>
+    <t>PIT</t>
+  </si>
+  <si>
+    <t>3072/CH-CR</t>
+  </si>
+  <si>
+    <t>Cantonal II</t>
+  </si>
+  <si>
+    <t>4864/OC-CR</t>
+  </si>
+  <si>
+    <t>PIV-APP</t>
+  </si>
+  <si>
+    <t>5823/OC-CR</t>
+  </si>
+  <si>
+    <t>San Carlos</t>
+  </si>
+  <si>
+    <t>4871/OC-CR</t>
+  </si>
+  <si>
+    <t>Seguridad Ciudadana</t>
+  </si>
+  <si>
+    <t>Migración</t>
+  </si>
+  <si>
+    <t>PIF</t>
+  </si>
+  <si>
+    <t>Educación</t>
+  </si>
+  <si>
+    <t>Cuidadados</t>
+  </si>
+  <si>
+    <t>Energía II</t>
+  </si>
+  <si>
     <t>Fecha de revisión</t>
   </si>
   <si>
@@ -1112,145 +1265,10 @@
     <t>nueva version para estructurar mejor la data preparando para futuro visor</t>
   </si>
   <si>
-    <t>PIT</t>
-  </si>
-  <si>
-    <t>Cantonal II</t>
-  </si>
-  <si>
-    <t>PIV-APP</t>
-  </si>
-  <si>
-    <t>San Carlos</t>
-  </si>
-  <si>
-    <t>Seguridad Ciudadana</t>
-  </si>
-  <si>
-    <t>Migración</t>
-  </si>
-  <si>
-    <t>PIF</t>
-  </si>
-  <si>
-    <t>Educación</t>
-  </si>
-  <si>
-    <t>Energía II</t>
-  </si>
-  <si>
-    <t>Cuidadados</t>
-  </si>
-  <si>
-    <t>Calificación Calculada</t>
-  </si>
-  <si>
-    <t>Calificación Validada</t>
-  </si>
-  <si>
-    <t>Programa de Infraestructura de Transporte</t>
-  </si>
-  <si>
-    <t>Programa Red Vial Cantonal II</t>
-  </si>
-  <si>
-    <t>Programa de Infraestructura Vial y promoción de Asociaciones Público-Privadas (APP)</t>
-  </si>
-  <si>
-    <t>Programa de Infraestructura Vial y Movilidad Urbana: conectividad resiliente</t>
-  </si>
-  <si>
-    <t>Programa de Seguridad Ciudadana y Prevención de Violencia</t>
-  </si>
-  <si>
-    <t>Programa Integral de Seguridad Ciudadana y Prevención de la Violencia para la Inclusión de Grupos Migrantes Vulnerables</t>
-  </si>
-  <si>
-    <t>Programa de Integración Fronteriza de Costa Rica</t>
-  </si>
-  <si>
-    <t>Mejora de la calidad del Sistema Educativo en Costa Rica</t>
-  </si>
-  <si>
-    <t>Apoyo al fortalecimiento y expansión del sistema nacional de cuidados de Costa Rica</t>
-  </si>
-  <si>
-    <t>Segundo Programa de Energía Renovable, Transmisión y Distribución de Electricidad</t>
-  </si>
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>OVIEDO BENAVIDES, GUSTAVO ALONSO</t>
-  </si>
-  <si>
-    <t>QUIROS SOLANO, FERNANDO ANDRES</t>
-  </si>
-  <si>
-    <t>VEGA GAMBOA, JORGE DANIEL</t>
-  </si>
-  <si>
-    <t>FARINACCIO, ALESSANDRO</t>
-  </si>
-  <si>
-    <t>ALVAREZ GONZALEZ, OSCAR ANDRES</t>
-  </si>
-  <si>
-    <t>Caminos cantonales rehabilitados</t>
-  </si>
-  <si>
-    <t>Rehabilitación de caminos (paquetes)</t>
-  </si>
-  <si>
-    <t>Puentes construidos o rehabilitados</t>
-  </si>
-  <si>
-    <t>Construcción de puentes (paquetes), rehabilitados (Incluye diseño adaptados a cambio climático).</t>
-  </si>
-  <si>
-    <t>Número de funcionarios municipales capacitados</t>
-  </si>
-  <si>
-    <t>Número de cantones con Planes Viales Quinquenales de conservación y desarrollo elaborados</t>
-  </si>
-  <si>
-    <t>Manuales de seguridad vial y gestión socioambiental elaborados</t>
-  </si>
-  <si>
-    <t>Sistema de Gestión de activos viales implementado</t>
-  </si>
-  <si>
-    <t>Cantones con intervención de seguridad vial</t>
-  </si>
-  <si>
-    <t>Mantenimiento rutinario por estándares realizado a través de microempresas</t>
-  </si>
-  <si>
-    <t>Evaluación Ex Post de resultados pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obras complementarias en el Tramo Central Sección Sucre – Abundancia </t>
-  </si>
-  <si>
-    <t>Pausado</t>
-  </si>
-  <si>
-    <t>Contratación para el diseño y construcción del Tramo Central de la Ruta Nacional no. 35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contratación para el diseño y construcción de la Punta Sur de la Ruta Nacional no. 35 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
-  </si>
-  <si>
-    <t>Contratación de para el diseño y construcción de los sistemas de iluminación vial para la Punta Norte de la RN No. 35 (Sección ciudad Quesada / Florencia)</t>
-  </si>
-  <si>
-    <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa. </t>
+    <t>implementa nuevo visor usando nueva estructura de datos</t>
+  </si>
+  <si>
+    <t>actualización de nombres y roles de equipo de proyecto usando nuevo agente de copilot</t>
   </si>
   <si>
     <t>clausulas</t>
@@ -1259,21 +1277,6 @@
     <t>generacion automática de filtros con base en csv generado por el dashboard de clausulas del banco</t>
   </si>
   <si>
-    <t>https://idbg.sharepoint.com/teams/ez-CR-L1157/_layouts/15/DocIdRedir.aspx?ID=EZIDB0003356-828744887-9</t>
-  </si>
-  <si>
-    <t>EZIDB0003356-828744887-9</t>
-  </si>
-  <si>
-    <t>https://idbg.sharepoint.com/teams/EZ-CR-LON/CR-L1065/_layouts/15/DocIdRedir.aspx?ID=EZIDB0000195-998400382-110</t>
-  </si>
-  <si>
-    <t>implementa nuevo visor usando nueva estructura de datos</t>
-  </si>
-  <si>
-    <t>actualización de nombres y roles de equipo de proyecto usando nuevo agente de copilot</t>
-  </si>
-  <si>
     <t>implementa nuevos tabs de clausulas vencidas y proximas a vencer generados automaticamente desde el csv del dashboard del banco</t>
   </si>
   <si>
@@ -1296,6 +1299,12 @@
   </si>
   <si>
     <t>actualiza codigo de colores para indicadores tecnicos segun guía de pmr</t>
+  </si>
+  <si>
+    <t>se actualiza estado</t>
+  </si>
+  <si>
+    <t>se actualiza estado y comentarios</t>
   </si>
 </sst>
 </file>
@@ -1468,7 +1477,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1692,30 +1701,39 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left style="medium">
+        <color rgb="FF000000"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
+      <top style="medium">
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top/>
@@ -1724,21 +1742,21 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
+      <right style="medium">
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left style="medium">
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1746,19 +1764,19 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
+      <right style="medium">
+        <color rgb="FF000000"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1768,7 +1786,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1978,8 +1996,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1990,13 +2008,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2346,25 +2376,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D60"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" style="61" customWidth="1"/>
     <col min="2" max="2" width="38" style="61" customWidth="1"/>
     <col min="3" max="3" width="42" style="61" customWidth="1"/>
     <col min="4" max="4" width="80" style="61" customWidth="1"/>
-    <col min="5" max="16384" width="8.85546875" style="61"/>
+    <col min="5" max="16384" width="8.88671875" style="61"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+    <row r="1" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-    </row>
-    <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+    </row>
+    <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
@@ -2378,7 +2408,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="62" t="s">
         <v>5</v>
       </c>
@@ -2392,7 +2422,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="62" t="s">
         <v>5</v>
       </c>
@@ -2406,7 +2436,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="62" t="s">
         <v>11</v>
       </c>
@@ -2420,7 +2450,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="62" t="s">
         <v>14</v>
       </c>
@@ -2434,7 +2464,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="62" t="s">
         <v>17</v>
       </c>
@@ -2448,7 +2478,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="62" t="s">
         <v>20</v>
       </c>
@@ -2462,7 +2492,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="62" t="s">
         <v>22</v>
       </c>
@@ -2476,7 +2506,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="62" t="s">
         <v>25</v>
       </c>
@@ -2490,7 +2520,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="62" t="s">
         <v>5</v>
       </c>
@@ -2504,7 +2534,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="62" t="s">
         <v>14</v>
       </c>
@@ -2518,7 +2548,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="62" t="s">
         <v>17</v>
       </c>
@@ -2532,7 +2562,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="62" t="s">
         <v>20</v>
       </c>
@@ -2546,7 +2576,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="62" t="s">
         <v>22</v>
       </c>
@@ -2560,7 +2590,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="62" t="s">
         <v>25</v>
       </c>
@@ -2574,7 +2604,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
         <v>41</v>
       </c>
@@ -2586,7 +2616,7 @@
       </c>
       <c r="D18" s="63"/>
     </row>
-    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
         <v>5</v>
       </c>
@@ -2600,7 +2630,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="62" t="s">
         <v>11</v>
       </c>
@@ -2614,7 +2644,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="62" t="s">
         <v>14</v>
       </c>
@@ -2628,7 +2658,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="62" t="s">
         <v>17</v>
       </c>
@@ -2642,7 +2672,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="62" t="s">
         <v>20</v>
       </c>
@@ -2656,7 +2686,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
         <v>22</v>
       </c>
@@ -2670,7 +2700,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="62" t="s">
         <v>25</v>
       </c>
@@ -2684,7 +2714,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="62" t="s">
         <v>58</v>
       </c>
@@ -2698,7 +2728,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="62" t="s">
         <v>5</v>
       </c>
@@ -2712,7 +2742,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="62" t="s">
         <v>14</v>
       </c>
@@ -2726,7 +2756,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="62" t="s">
         <v>17</v>
       </c>
@@ -2740,7 +2770,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="62" t="s">
         <v>20</v>
       </c>
@@ -2754,7 +2784,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="62" t="s">
         <v>22</v>
       </c>
@@ -2768,7 +2798,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="62" t="s">
         <v>41</v>
       </c>
@@ -2782,7 +2812,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="62" t="s">
         <v>58</v>
       </c>
@@ -2796,7 +2826,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="62" t="s">
         <v>5</v>
       </c>
@@ -2810,7 +2840,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="62" t="s">
         <v>5</v>
       </c>
@@ -2824,7 +2854,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="62" t="s">
         <v>11</v>
       </c>
@@ -2838,7 +2868,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="62" t="s">
         <v>14</v>
       </c>
@@ -2852,7 +2882,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="62" t="s">
         <v>17</v>
       </c>
@@ -2866,7 +2896,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="62" t="s">
         <v>20</v>
       </c>
@@ -2880,7 +2910,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="62" t="s">
         <v>22</v>
       </c>
@@ -2894,7 +2924,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="62" t="s">
         <v>25</v>
       </c>
@@ -2908,7 +2938,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="62" t="s">
         <v>58</v>
       </c>
@@ -2922,7 +2952,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="62" t="s">
         <v>5</v>
       </c>
@@ -2936,7 +2966,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="62" t="s">
         <v>14</v>
       </c>
@@ -2950,7 +2980,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="62" t="s">
         <v>17</v>
       </c>
@@ -2964,7 +2994,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="62" t="s">
         <v>20</v>
       </c>
@@ -2978,7 +3008,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="62" t="s">
         <v>58</v>
       </c>
@@ -2992,7 +3022,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="62" t="s">
         <v>5</v>
       </c>
@@ -3006,7 +3036,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="62" t="s">
         <v>11</v>
       </c>
@@ -3020,7 +3050,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="62" t="s">
         <v>14</v>
       </c>
@@ -3034,7 +3064,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="62" t="s">
         <v>17</v>
       </c>
@@ -3048,7 +3078,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="62" t="s">
         <v>20</v>
       </c>
@@ -3062,7 +3092,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="62" t="s">
         <v>22</v>
       </c>
@@ -3076,7 +3106,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="62" t="s">
         <v>25</v>
       </c>
@@ -3090,7 +3120,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="62" t="s">
         <v>5</v>
       </c>
@@ -3104,7 +3134,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="62" t="s">
         <v>11</v>
       </c>
@@ -3115,10 +3145,10 @@
         <v>123</v>
       </c>
       <c r="D56" s="63" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="62" t="s">
         <v>17</v>
       </c>
@@ -3126,13 +3156,13 @@
         <v>120</v>
       </c>
       <c r="C57" s="63" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D57" s="63" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="62" t="s">
         <v>20</v>
       </c>
@@ -3140,13 +3170,13 @@
         <v>120</v>
       </c>
       <c r="C58" s="63" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D58" s="63" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="62" t="s">
         <v>58</v>
       </c>
@@ -3154,13 +3184,13 @@
         <v>6</v>
       </c>
       <c r="C59" s="63" t="s">
-        <v>388</v>
+        <v>128</v>
       </c>
       <c r="D59" s="63" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="62" t="s">
         <v>25</v>
       </c>
@@ -3186,33 +3216,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:K21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.5703125" customWidth="1"/>
-    <col min="3" max="3" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2" s="6">
         <v>46162</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>5</v>
@@ -3242,73 +3272,73 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="K6" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>130</v>
-      </c>
       <c r="F7" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H7" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
         <v>138</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -3318,43 +3348,43 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -3362,286 +3392,286 @@
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>361</v>
+        <v>156</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>361</v>
+        <v>156</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>361</v>
+        <v>156</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>361</v>
+        <v>156</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>364</v>
+        <v>161</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J14" s="5"/>
       <c r="K14" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>363</v>
+        <v>165</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>363</v>
+        <v>165</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>362</v>
+        <v>171</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>362</v>
+        <v>171</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>362</v>
+        <v>171</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>363</v>
+        <v>165</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>362</v>
+        <v>171</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="G19" s="5" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
@@ -3649,16 +3679,16 @@
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="J20" s="5"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>160</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
@@ -3676,715 +3706,713 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:G41"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" customWidth="1"/>
-    <col min="3" max="3" width="46.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="39.7109375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="37.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="69.28515625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="2"/>
+    <col min="3" max="3" width="46.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="39.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="37.109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="38" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
       <c r="G4" s="16" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D5" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="G5" s="20" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D6" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="G6" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" s="20" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D7" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="E7" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>384</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E8" s="25"/>
       <c r="F8" s="25"/>
       <c r="G8" s="26" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G10" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="D10" s="21" t="s">
-        <v>191</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="G10" s="20" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" ht="58.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="2:7" ht="58.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="27" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E11" s="30"/>
       <c r="F11" s="30"/>
       <c r="G11" s="31" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="D12" s="32" t="s">
-        <v>191</v>
-      </c>
       <c r="E12" s="13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="27" t="s">
         <v>22</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="33" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="17" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="27" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="28" t="s">
-        <v>217</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="E17" s="28" t="s">
+      <c r="C17" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="G17" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="F17" s="30"/>
-      <c r="G17" s="31" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" ht="137.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="12" t="s">
+    </row>
+    <row r="18" spans="2:7" ht="137.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="15" t="s">
-        <v>219</v>
-      </c>
-      <c r="D18" s="32" t="s">
-        <v>378</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" ht="137.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="12" t="s">
+      <c r="C18" s="72" t="s">
+        <v>223</v>
+      </c>
+      <c r="D18" s="81" t="s">
+        <v>224</v>
+      </c>
+      <c r="E18" s="73" t="s">
+        <v>225</v>
+      </c>
+      <c r="F18" s="73" t="s">
+        <v>226</v>
+      </c>
+      <c r="G18" s="82" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="137.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>378</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="20"/>
-    </row>
-    <row r="20" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="17" t="s">
+      <c r="C19" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="D19" s="81" t="s">
+        <v>224</v>
+      </c>
+      <c r="E19" s="73" t="s">
+        <v>225</v>
+      </c>
+      <c r="F19" s="73"/>
+      <c r="G19" s="82"/>
+    </row>
+    <row r="20" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="74" t="s">
         <v>25</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>380</v>
+        <v>230</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="G20" s="20" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="G20" s="83" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" ht="81" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="D21" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>382</v>
-      </c>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-    </row>
-    <row r="22" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="71" t="s">
+      <c r="C21" s="77" t="s">
+        <v>233</v>
+      </c>
+      <c r="D21" s="78" t="s">
+        <v>188</v>
+      </c>
+      <c r="E21" s="79" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="79"/>
+      <c r="G21" s="80"/>
+    </row>
+    <row r="22" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="25" t="s">
-        <v>370</v>
-      </c>
-      <c r="D22" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="F22" s="25"/>
-      <c r="G22" s="72"/>
-    </row>
-    <row r="23" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="73" t="s">
+      <c r="C22" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="G22" s="75"/>
+    </row>
+    <row r="23" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>371</v>
+        <v>237</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E23" s="18"/>
-      <c r="G23" s="74"/>
-    </row>
-    <row r="24" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="73" t="s">
+      <c r="G23" s="75"/>
+    </row>
+    <row r="24" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>372</v>
+        <v>238</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E24" s="18"/>
-      <c r="G24" s="74"/>
-    </row>
-    <row r="25" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="73" t="s">
+      <c r="G24" s="75"/>
+    </row>
+    <row r="25" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>373</v>
+        <v>239</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E25" s="18"/>
-      <c r="G25" s="74"/>
-    </row>
-    <row r="26" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="73" t="s">
+      <c r="G25" s="75"/>
+    </row>
+    <row r="26" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>374</v>
+        <v>240</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E26" s="18"/>
-      <c r="G26" s="74"/>
-    </row>
-    <row r="27" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="73" t="s">
+      <c r="G26" s="75"/>
+    </row>
+    <row r="27" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>375</v>
+        <v>241</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E27" s="18"/>
-      <c r="G27" s="74"/>
-    </row>
-    <row r="28" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="73" t="s">
+      <c r="G27" s="75"/>
+    </row>
+    <row r="28" spans="2:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>368</v>
+        <v>242</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>369</v>
+        <v>243</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="G28" s="74"/>
-    </row>
-    <row r="29" spans="2:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="75" t="s">
+        <v>244</v>
+      </c>
+      <c r="G28" s="75"/>
+    </row>
+    <row r="29" spans="2:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="76" t="s">
-        <v>366</v>
-      </c>
-      <c r="D29" s="77" t="s">
-        <v>189</v>
-      </c>
-      <c r="E29" s="78" t="s">
-        <v>367</v>
-      </c>
-      <c r="F29" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="G29" s="79" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" ht="99" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="77" t="s">
+        <v>245</v>
+      </c>
+      <c r="D29" s="78" t="s">
+        <v>188</v>
+      </c>
+      <c r="E29" s="79" t="s">
+        <v>246</v>
+      </c>
+      <c r="F29" s="79" t="s">
+        <v>244</v>
+      </c>
+      <c r="G29" s="80" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="17" t="s">
         <v>20</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>227</v>
+        <v>248</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>228</v>
+        <v>249</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>229</v>
+        <v>250</v>
       </c>
       <c r="G30" s="20" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="17" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>227</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>189</v>
+        <v>248</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>202</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>231</v>
+        <v>252</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="104.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="17" t="s">
         <v>20</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>233</v>
+        <v>254</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>234</v>
+        <v>255</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>235</v>
+        <v>256</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>20</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>236</v>
+        <v>257</v>
       </c>
       <c r="D33" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="G33" s="39" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" ht="100.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>189</v>
-      </c>
       <c r="E34" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="F34" s="82" t="s">
-        <v>243</v>
+        <v>263</v>
+      </c>
+      <c r="F34" s="86" t="s">
+        <v>264</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="17" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>245</v>
+        <v>266</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>246</v>
-      </c>
-      <c r="F35" s="83"/>
+        <v>267</v>
+      </c>
+      <c r="F35" s="87"/>
       <c r="G35" s="20" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="17" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>245</v>
+        <v>266</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>248</v>
-      </c>
-      <c r="F36" s="83"/>
+        <v>269</v>
+      </c>
+      <c r="F36" s="87"/>
       <c r="G36" s="20" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" ht="195" customHeight="1" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" ht="195" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
         <v>5</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>249</v>
+        <v>270</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="38" spans="2:7" ht="188.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="17" t="s">
         <v>5</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>254</v>
+        <v>275</v>
       </c>
       <c r="F38" s="18" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="39" spans="2:7" ht="193.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" ht="193.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="17" t="s">
         <v>5</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="D39" s="21" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>257</v>
+        <v>278</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
       <c r="G39" s="20" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="40" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="17" t="s">
         <v>5</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F40" s="18" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="G40" s="20" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="41" spans="2:7" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="27" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="30" t="s">
-        <v>262</v>
+        <v>283</v>
       </c>
       <c r="D41" s="29" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E41" s="30"/>
       <c r="F41" s="28" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>263</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -4399,134 +4427,134 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:Q14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="57.140625" customWidth="1"/>
-    <col min="4" max="5" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="57.109375" customWidth="1"/>
+    <col min="4" max="5" width="19.33203125" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="11.85546875" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" customWidth="1"/>
-    <col min="10" max="11" width="10.5703125" customWidth="1"/>
-    <col min="12" max="12" width="7.85546875" customWidth="1"/>
-    <col min="13" max="13" width="62.42578125" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" customWidth="1"/>
+    <col min="10" max="11" width="10.5546875" customWidth="1"/>
+    <col min="12" max="12" width="7.88671875" customWidth="1"/>
+    <col min="13" max="13" width="62.44140625" customWidth="1"/>
     <col min="14" max="14" width="45" customWidth="1"/>
-    <col min="16" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:17" ht="21" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="60" t="s">
-        <v>264</v>
+        <v>285</v>
       </c>
       <c r="C2" s="60"/>
     </row>
-    <row r="4" spans="2:17" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="69" t="s">
-        <v>172</v>
+        <v>286</v>
       </c>
       <c r="C4" s="69" t="s">
-        <v>360</v>
+        <v>287</v>
       </c>
       <c r="D4" s="68" t="s">
-        <v>348</v>
+        <v>288</v>
       </c>
       <c r="E4" s="58" t="s">
-        <v>349</v>
+        <v>289</v>
       </c>
       <c r="F4" s="59" t="s">
-        <v>265</v>
+        <v>290</v>
       </c>
       <c r="G4" s="59" t="s">
-        <v>266</v>
+        <v>291</v>
       </c>
       <c r="H4" s="59" t="s">
-        <v>267</v>
+        <v>292</v>
       </c>
       <c r="I4" s="59" t="s">
-        <v>268</v>
+        <v>293</v>
       </c>
       <c r="J4" s="59" t="s">
-        <v>269</v>
+        <v>294</v>
       </c>
       <c r="K4" s="59" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
       <c r="L4" s="59" t="s">
-        <v>271</v>
+        <v>296</v>
       </c>
       <c r="M4" s="58" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="N4" s="58" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="5" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="70" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>350</v>
+        <v>299</v>
       </c>
       <c r="D5" s="64" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="E5" s="41" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="F5" s="45">
         <v>0.77</v>
       </c>
       <c r="G5" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="H5" s="47">
         <v>1</v>
       </c>
       <c r="I5" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="J5" s="47">
         <v>1.01</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="L5" s="42">
         <v>2</v>
       </c>
       <c r="M5" s="40" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="N5" s="40" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="6" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="70" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>351</v>
+        <v>304</v>
       </c>
       <c r="D6" s="65" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F6" s="49">
         <v>0.97</v>
       </c>
       <c r="G6" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="H6" s="47">
         <v>0.95</v>
       </c>
       <c r="I6" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="J6" s="47">
         <v>1.05</v>
@@ -4538,24 +4566,24 @@
         <v>3</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="N6" s="40" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="7" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>352</v>
+        <v>307</v>
       </c>
       <c r="D7" s="65" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F7" s="49">
         <v>0.65000000000000191</v>
@@ -4573,30 +4601,30 @@
         <v>1.0760758704453901</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="L7" s="42">
         <v>2</v>
       </c>
       <c r="M7" s="40" t="s">
-        <v>280</v>
+        <v>308</v>
       </c>
       <c r="N7" s="40" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="70" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>353</v>
+        <v>310</v>
       </c>
       <c r="D8" s="65" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F8" s="51">
         <v>0.04</v>
@@ -4614,71 +4642,71 @@
         <v>1</v>
       </c>
       <c r="K8" s="44" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="L8" s="42">
         <v>2</v>
       </c>
       <c r="M8" s="40" t="s">
-        <v>282</v>
+        <v>311</v>
       </c>
       <c r="N8" s="40" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="9" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="70" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>354</v>
+        <v>313</v>
       </c>
       <c r="D9" s="64" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F9" s="49">
         <v>0.65</v>
       </c>
       <c r="G9" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="H9" s="50">
         <v>0.75</v>
       </c>
       <c r="I9" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="J9" s="50">
         <v>0.74</v>
       </c>
       <c r="K9" s="44" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="L9" s="42">
         <v>2</v>
       </c>
       <c r="M9" s="40" t="s">
-        <v>284</v>
+        <v>314</v>
       </c>
       <c r="N9" s="40" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="70" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>355</v>
+        <v>316</v>
       </c>
       <c r="D10" s="66" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="E10" s="53" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="F10" s="49">
         <v>0.38000000000000012</v>
@@ -4696,42 +4724,42 @@
         <v>2.737091349830477</v>
       </c>
       <c r="K10" s="44" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="L10" s="42">
         <v>2</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>287</v>
+        <v>318</v>
       </c>
       <c r="N10" s="40" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="70" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>356</v>
+        <v>320</v>
       </c>
       <c r="D11" s="65" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F11" s="54">
         <v>1</v>
       </c>
       <c r="G11" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="H11" s="47">
         <v>0.95</v>
       </c>
       <c r="I11" s="46" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="J11" s="47">
         <v>0.9</v>
@@ -4743,24 +4771,24 @@
         <v>3</v>
       </c>
       <c r="M11" s="40" t="s">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="N11" s="40" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="12" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="70" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>357</v>
+        <v>321</v>
       </c>
       <c r="D12" s="64" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F12" s="41"/>
       <c r="G12" s="41"/>
@@ -4770,24 +4798,24 @@
       <c r="K12" s="41"/>
       <c r="L12" s="41"/>
       <c r="M12" s="55" t="s">
-        <v>289</v>
+        <v>322</v>
       </c>
       <c r="N12" s="40" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="70" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="D13" s="67" t="s">
-        <v>292</v>
+        <v>326</v>
       </c>
       <c r="E13" s="56" t="s">
-        <v>292</v>
+        <v>326</v>
       </c>
       <c r="F13" s="56"/>
       <c r="G13" s="56"/>
@@ -4797,24 +4825,24 @@
       <c r="K13" s="56"/>
       <c r="L13" s="56"/>
       <c r="M13" s="55" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="N13" s="40" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="70" t="s">
         <v>58</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>359</v>
+        <v>328</v>
       </c>
       <c r="D14" s="65" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -4824,10 +4852,10 @@
       <c r="K14" s="43"/>
       <c r="L14" s="43"/>
       <c r="M14" s="55" t="s">
-        <v>294</v>
+        <v>329</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
       <c r="P14" s="57"/>
       <c r="Q14" s="57"/>
@@ -4841,142 +4869,142 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F546759E-1E7A-4FBA-BCE7-8747DD03CB19}">
   <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>175</v>
+        <v>331</v>
       </c>
       <c r="D2" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="E2" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>174</v>
+        <v>333</v>
       </c>
       <c r="D3" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="E3" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="E4" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>335</v>
       </c>
       <c r="D5" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E5" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>177</v>
+        <v>337</v>
       </c>
       <c r="D6" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E6" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>173</v>
+        <v>339</v>
       </c>
       <c r="D7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E7" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E8" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E9" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E10" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="D11" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E11" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>58</v>
       </c>
       <c r="D12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E12" t="s">
-        <v>359</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -4986,514 +5014,514 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:E43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:E45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="4" max="4" width="36.44140625" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>296</v>
+        <v>346</v>
       </c>
       <c r="C2" t="s">
-        <v>297</v>
+        <v>347</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C3" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C4" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C5" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C6" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C7" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C8" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C9" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D9" t="s">
         <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C10" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C11" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D11" t="s">
         <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C12" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C13" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D13" t="s">
-        <v>312</v>
+        <v>362</v>
       </c>
       <c r="E13" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C14" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D14" t="s">
         <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C15" t="s">
-        <v>314</v>
+        <v>364</v>
       </c>
       <c r="D15" t="s">
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C16" t="s">
-        <v>314</v>
+        <v>364</v>
       </c>
       <c r="D16" t="s">
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C17" t="s">
-        <v>314</v>
+        <v>364</v>
       </c>
       <c r="D17" t="s">
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="C18" t="s">
-        <v>318</v>
+        <v>368</v>
       </c>
       <c r="D18" t="s">
         <v>17</v>
       </c>
       <c r="E18" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="8">
         <v>46092</v>
       </c>
       <c r="C19" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="8">
         <v>46092</v>
       </c>
       <c r="C20" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D20" t="s">
-        <v>312</v>
+        <v>362</v>
       </c>
       <c r="E20" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="8">
         <v>46092</v>
       </c>
       <c r="C21" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
       </c>
       <c r="E21" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="8">
         <v>46092</v>
       </c>
       <c r="C22" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D22" t="s">
         <v>17</v>
       </c>
       <c r="E22" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="8">
         <v>46092</v>
       </c>
       <c r="C23" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D23" t="s">
         <v>20</v>
       </c>
       <c r="E23" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="8">
         <v>46092</v>
       </c>
       <c r="C24" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D24" t="s">
         <v>41</v>
       </c>
       <c r="E24" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="8">
         <v>46092</v>
       </c>
       <c r="C25" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D25" t="s">
         <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="8">
         <v>46119</v>
       </c>
       <c r="C26" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="E26" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="8">
         <v>46119</v>
       </c>
       <c r="C27" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D27" t="s">
         <v>20</v>
       </c>
       <c r="E27" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="8">
         <v>46119</v>
       </c>
       <c r="C28" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D28" t="s">
         <v>17</v>
       </c>
       <c r="E28" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="8">
         <v>46119</v>
       </c>
       <c r="C29" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="D29" t="s">
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="8">
         <v>46121</v>
       </c>
       <c r="C30" t="s">
-        <v>326</v>
+        <v>376</v>
       </c>
       <c r="D30" t="s">
-        <v>327</v>
+        <v>377</v>
       </c>
       <c r="E30" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="8">
         <v>46121</v>
       </c>
       <c r="C31" t="s">
-        <v>329</v>
+        <v>379</v>
       </c>
       <c r="D31" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
       <c r="E31" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="8">
         <v>46126</v>
       </c>
       <c r="C32" t="s">
-        <v>332</v>
+        <v>382</v>
       </c>
       <c r="D32" t="s">
-        <v>333</v>
+        <v>383</v>
       </c>
       <c r="E32" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="8">
         <v>46134</v>
       </c>
       <c r="C33" t="s">
-        <v>335</v>
+        <v>385</v>
       </c>
       <c r="E33" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="8">
         <v>46134</v>
       </c>
       <c r="C34" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="E34" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="8">
         <v>46142</v>
       </c>
       <c r="C35" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="E35" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="8">
         <v>46160</v>
       </c>
       <c r="C36" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="E36" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B37" s="8">
         <v>46169</v>
       </c>
       <c r="C37" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="E37" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B38" s="8">
         <v>46170</v>
       </c>
       <c r="C38" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="E38" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39" s="8">
         <v>46170</v>
       </c>
@@ -5504,12 +5532,12 @@
         <v>394</v>
       </c>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B40" s="8">
         <v>46170</v>
       </c>
       <c r="C40" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="D40" t="s">
         <v>58</v>
@@ -5518,29 +5546,29 @@
         <v>395</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B41" s="8">
         <v>46171</v>
       </c>
       <c r="C41" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="E41" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B42" s="8">
         <v>46171</v>
       </c>
       <c r="C42" t="s">
-        <v>307</v>
+        <v>357</v>
       </c>
       <c r="E42" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B43" s="8">
         <v>46171</v>
       </c>
@@ -5549,6 +5577,34 @@
       </c>
       <c r="E43" t="s">
         <v>399</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B44" s="8">
+        <v>46171</v>
+      </c>
+      <c r="C44" t="s">
+        <v>376</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B45" s="8">
+        <v>46171</v>
+      </c>
+      <c r="C45" t="s">
+        <v>376</v>
+      </c>
+      <c r="D45" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eliminar columna G "Resultado asociado" de hoja productos criticos
La columna no es leída ni utilizada en ningún lugar del visor.
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3270" yWindow="630" windowWidth="20460" windowHeight="14490" tabRatio="819" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="documentos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="equipo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="productos criticos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PMR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="datos_ops" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resultados" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="productos_resultados" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="change log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="documentos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="equipo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="productos criticos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PMR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="datos_ops" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="resultados" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="productos_resultados" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="change log" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$3:$D$60</definedName>
@@ -3301,7 +3301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G41"/>
+  <dimension ref="B2:F41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="85" min="1" max="1"/>
@@ -3348,11 +3348,6 @@
           <t>Riesgos/Comentarios</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>Resultado asociado</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="28.95" customHeight="1" s="89">
       <c r="B4" s="12" t="inlineStr">
@@ -3372,11 +3367,6 @@
       </c>
       <c r="E4" s="15" t="n"/>
       <c r="F4" s="15" t="n"/>
-      <c r="G4" s="16" t="inlineStr">
-        <is>
-          <t>1.1 Homicidios en distritos priorizados  [tasa] y 1.2 Asaltos en distritos priorizados [tasa]</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="28.95" customHeight="1" s="89">
       <c r="B5" s="17" t="inlineStr">
@@ -3394,11 +3384,6 @@
           <t>En tiempo</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Homicidios en distritos priorizados  [tasa] y 1.2 Asaltos en distritos priorizados [tasa]</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="28.95" customHeight="1" s="89">
       <c r="B6" s="17" t="inlineStr">
@@ -3426,11 +3411,6 @@
           <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Homicidios en distritos priorizados  [tasa] y 1.2 Asaltos en distritos priorizados [tasa]</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="43.2" customHeight="1" s="89">
       <c r="B7" s="17" t="inlineStr">
@@ -3458,11 +3438,6 @@
           <t xml:space="preserve">Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa. </t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Homicidios en distritos priorizados  [tasa] y 1.2 Asaltos en distritos priorizados [tasa]</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="57.6" customHeight="1" s="89">
       <c r="B8" s="22" t="inlineStr">
@@ -3482,11 +3457,6 @@
       </c>
       <c r="E8" s="25" t="n"/>
       <c r="F8" s="25" t="n"/>
-      <c r="G8" s="26" t="inlineStr">
-        <is>
-          <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="57.6" customHeight="1" s="89">
       <c r="B9" s="17" t="inlineStr">
@@ -3504,11 +3474,6 @@
           <t>Logrado</t>
         </is>
       </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="57.6" customHeight="1" s="89">
       <c r="B10" s="17" t="inlineStr">
@@ -3536,11 +3501,6 @@
           <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="58.2" customHeight="1" s="89" thickBot="1">
       <c r="B11" s="27" t="inlineStr">
@@ -3560,11 +3520,6 @@
       </c>
       <c r="E11" s="30" t="n"/>
       <c r="F11" s="30" t="n"/>
-      <c r="G11" s="31" t="inlineStr">
-        <is>
-          <t>2.1 Exclusión escolar (fuera del sistema educativo) de jóvenes entre 12 y 17 años que participan en los CCP [porcentaje] y 2.2 Proporción de aprehensiones de jóvenes menores de edad en los distritos de influencia de los CCP con respecto al total país [porcentaje]</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="43.2" customHeight="1" s="89" thickBot="1">
       <c r="B12" s="12" t="inlineStr">
@@ -3592,11 +3547,6 @@
           <t>Capacidad de presupuestación de fondos limita el ritmo de contratación de personal de apoyo</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>1.1 Tiempo promedio entre solicitud y entrevista para el trámite de obtención del status de refugiado [años] y 1.4 Porcentaje de solicitudes de protección especial complementaria que son resueltas en un plazo menor a un año [%]</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="43.95" customHeight="1" s="89" thickBot="1">
       <c r="B13" s="27" t="inlineStr">
@@ -3624,11 +3574,6 @@
           <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
-      <c r="G13" s="31" t="inlineStr">
-        <is>
-          <t>1.1 Tiempo promedio entre solicitud y entrevista para el trámite de obtención del status de refugiado [años] y 1.4 Porcentaje de solicitudes de protección especial complementaria que son resueltas en un plazo menor a un año [%]</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="29.4" customHeight="1" s="89" thickBot="1">
       <c r="B14" s="33" t="inlineStr">
@@ -3656,11 +3601,6 @@
           <t>El proceso de adquisición no ha iniciado</t>
         </is>
       </c>
-      <c r="G14" s="37" t="inlineStr">
-        <is>
-          <t>1.2 Porcentaje promedio de reacciones xenófobas a tweets de cuentas migratorias institucionales [%]</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="28.95" customHeight="1" s="89">
       <c r="B15" s="12" t="inlineStr">
@@ -3688,11 +3628,6 @@
           <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>1.3 Ratio de migrantes que asisten de manera recurrente a los centros de acogida y participan en actividades para la prevención social de la violencia [ratio]</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="28.95" customHeight="1" s="89">
       <c r="B16" s="17" t="inlineStr">
@@ -3715,11 +3650,6 @@
           <t>Formadores expertos en prevención de tráfico ilícito (3 consultores individuales)</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t>1.3 Ratio de migrantes que asisten de manera recurrente a los centros de acogida y participan en actividades para la prevención social de la violencia [ratio]</t>
-        </is>
-      </c>
     </row>
     <row r="17" ht="29.4" customHeight="1" s="89">
       <c r="B17" s="17" t="inlineStr">
@@ -3742,11 +3672,6 @@
           <t>Gestor metodológico y Facilitadores de formación en CCP (cons. Individuales)</t>
         </is>
       </c>
-      <c r="G17" s="20" t="inlineStr">
-        <is>
-          <t>1.3 Ratio de migrantes que asisten de manera recurrente a los centros de acogida y participan en actividades para la prevención social de la violencia [ratio]</t>
-        </is>
-      </c>
     </row>
     <row r="18" ht="137.25" customHeight="1" s="89">
       <c r="B18" s="71" t="inlineStr">
@@ -3774,14 +3699,6 @@
           <t>En análisis por FMP y TSP junto con el OE sobre siguiente estado del proceso: declaración de infructuoso, cancelación, o nueva fuente de financiamiento.</t>
         </is>
       </c>
-      <c r="G18" s="82" t="inlineStr">
-        <is>
-          <t>1.1 Tiempo promedio de recorrido por vehículo en el tramo Florencia RN-1
-1.2 Costo de operación vehicular en el tramo de Florencia RN-1 (vehículo liviano)
-1.3. Nivel de seguridad vial (cantidad de estrellas mediante la metodología de iRAP) de la RN-35
-1.5. Sitios de la vía en el tramo de Abundancia Sifón (Tramo Central) afectados por inundaciones debido a precipitaciones con un período de retorno de 100 años.</t>
-        </is>
-      </c>
     </row>
     <row r="19" ht="137.25" customHeight="1" s="89">
       <c r="B19" s="71" t="inlineStr">
@@ -3805,7 +3722,6 @@
         </is>
       </c>
       <c r="F19" s="73" t="n"/>
-      <c r="G19" s="82" t="n"/>
     </row>
     <row r="20" ht="81" customHeight="1" s="89">
       <c r="B20" s="74" t="inlineStr">
@@ -3834,13 +3750,6 @@
 Lote 2 firmado.</t>
         </is>
       </c>
-      <c r="G20" s="83" t="inlineStr">
-        <is>
-          <t>1.1 Tiempo promedio de recorrido por vehículo en el tramo Florencia RN-1
-1.2 Costo de operación vehicular en el tramo de Florencia RN-1 (vehículo liviano)
-1.3. Nivel de seguridad vial (cantidad de estrellas mediante la metodología de iRAP) de la RN-35</t>
-        </is>
-      </c>
     </row>
     <row r="21" ht="81" customHeight="1" s="89">
       <c r="B21" s="76" t="inlineStr">
@@ -3864,7 +3773,6 @@
         </is>
       </c>
       <c r="F21" s="79" t="n"/>
-      <c r="G21" s="80" t="n"/>
     </row>
     <row r="22" ht="42.75" customHeight="1" s="89">
       <c r="B22" s="74" t="inlineStr">
@@ -3887,7 +3795,6 @@
           <t>Consultor individual que realice el PCR de operación</t>
         </is>
       </c>
-      <c r="G22" s="75" t="n"/>
     </row>
     <row r="23" ht="42.75" customHeight="1" s="89">
       <c r="B23" s="74" t="inlineStr">
@@ -3906,7 +3813,6 @@
         </is>
       </c>
       <c r="E23" s="18" t="n"/>
-      <c r="G23" s="75" t="n"/>
     </row>
     <row r="24" ht="42.75" customHeight="1" s="89">
       <c r="B24" s="74" t="inlineStr">
@@ -3925,7 +3831,6 @@
         </is>
       </c>
       <c r="E24" s="18" t="n"/>
-      <c r="G24" s="75" t="n"/>
     </row>
     <row r="25" ht="42.75" customHeight="1" s="89">
       <c r="B25" s="74" t="inlineStr">
@@ -3944,7 +3849,6 @@
         </is>
       </c>
       <c r="E25" s="18" t="n"/>
-      <c r="G25" s="75" t="n"/>
     </row>
     <row r="26" ht="42.75" customHeight="1" s="89">
       <c r="B26" s="74" t="inlineStr">
@@ -3963,7 +3867,6 @@
         </is>
       </c>
       <c r="E26" s="18" t="n"/>
-      <c r="G26" s="75" t="n"/>
     </row>
     <row r="27" ht="42.75" customHeight="1" s="89">
       <c r="B27" s="74" t="inlineStr">
@@ -3982,7 +3885,6 @@
         </is>
       </c>
       <c r="E27" s="18" t="n"/>
-      <c r="G27" s="75" t="n"/>
     </row>
     <row r="28" ht="42.75" customHeight="1" s="89">
       <c r="B28" s="74" t="inlineStr">
@@ -4010,7 +3912,6 @@
           <t>Evaluación Ex Post de resultados pendiente</t>
         </is>
       </c>
-      <c r="G28" s="75" t="n"/>
     </row>
     <row r="29" ht="80.25" customHeight="1" s="89">
       <c r="B29" s="76" t="inlineStr">
@@ -4038,13 +3939,6 @@
           <t>Evaluación Ex Post de resultados pendiente</t>
         </is>
       </c>
-      <c r="G29" s="80" t="inlineStr">
-        <is>
-          <t>1.1 Densidad de vías cantonales en buen estado
-2.1 1 Costos de operación vehicular en tramos que pasan de Lastre o Tierra a Tratamiento Bituminoso Simple (TBS)
-3.1 Costos de viaje en tramos que pasan de Lastre o Tierra a Tratamiento Bituminoso Simple (TBS)</t>
-        </is>
-      </c>
     </row>
     <row r="30" ht="99" customHeight="1" s="89">
       <c r="B30" s="17" t="inlineStr">
@@ -4073,13 +3967,6 @@
 En proceso de finalizar expropiaciones. </t>
         </is>
       </c>
-      <c r="G30" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Costos de operación vehicular ponderado en los sitios de las OBIS en el tramo San José – San Ramón. 
-2.1 Tiempo de viaje promedio de los vehículos que circulan por el tramo San José -San Ramón en la hora de mayor congestión
-3.1 Sumario de toneladas retenidas (ahorro) de emisiones de CO2 generadas por los vehículos que circulan en el tramo San José – San Ramón.</t>
-        </is>
-      </c>
     </row>
     <row r="31" ht="86.40000000000001" customHeight="1" s="89">
       <c r="B31" s="17" t="inlineStr">
@@ -4107,13 +3994,6 @@
           <t>En revisión enmienda al contrato por ajustes en el diseño final que implicaría aumento de alcance, costo y tiempo.</t>
         </is>
       </c>
-      <c r="G31" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Costos de operación vehicular ponderado en los sitios de las OBIS en el tramo San José – San Ramón. 
-2.1 Tiempo de viaje promedio de los vehículos que circulan por el tramo San José -San Ramón en la hora de mayor congestión
-3.1 Sumario de toneladas retenidas (ahorro) de emisiones de CO2 generadas por los vehículos que circulan en el tramo San José – San Ramón.</t>
-        </is>
-      </c>
     </row>
     <row r="32" ht="104.25" customHeight="1" s="89">
       <c r="B32" s="17" t="inlineStr">
@@ -4143,13 +4023,6 @@
 Estimado por US$2.5 millones.</t>
         </is>
       </c>
-      <c r="G32" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Costos de operación vehicular ponderado en los sitios de las OBIS en el tramo San José – San Ramón. 
-2.1 Tiempo de viaje promedio de los vehículos que circulan por el tramo San José -San Ramón en la hora de mayor congestión
-3.1 Sumario de toneladas retenidas (ahorro) de emisiones de CO2 generadas por los vehículos que circulan en el tramo San José – San Ramón.</t>
-        </is>
-      </c>
     </row>
     <row r="33" ht="46.5" customHeight="1" s="89" thickBot="1">
       <c r="B33" s="17" t="inlineStr">
@@ -4177,11 +4050,6 @@
           <t>Proyecto #2 aún no definido por el OE.</t>
         </is>
       </c>
-      <c r="G33" s="39" t="inlineStr">
-        <is>
-          <t>4.1 Proyectos de Obras Viales Estructurados bajo la modalidad de APP</t>
-        </is>
-      </c>
     </row>
     <row r="34" ht="100.95" customHeight="1" s="89">
       <c r="B34" s="12" t="inlineStr">
@@ -4210,12 +4078,6 @@
           <t xml:space="preserve">Se debe actualizar la planificación para validarla mediante un taller de arranque, junto con la Unidad Ejecutora y la Jefe de Equipo. </t>
         </is>
       </c>
-      <c r="G34" s="16" t="inlineStr">
-        <is>
-          <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable.
-1. 2 Número total de espacios públicos que disponen de sistema saneamiento nuevos o mejorados</t>
-        </is>
-      </c>
     </row>
     <row r="35" ht="43.2" customHeight="1" s="89">
       <c r="B35" s="17" t="inlineStr">
@@ -4238,11 +4100,6 @@
           <t>Diseño de la obra e inspección (sistemas de saneamiento).</t>
         </is>
       </c>
-      <c r="G35" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable.</t>
-        </is>
-      </c>
     </row>
     <row r="36" ht="43.95" customHeight="1" s="89" thickBot="1">
       <c r="B36" s="17" t="inlineStr">
@@ -4265,11 +4122,6 @@
           <t>Sistemas de Saneamiento en hogares rurales (construcción de la obra)</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr">
-        <is>
-          <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable.</t>
-        </is>
-      </c>
     </row>
     <row r="37" ht="195" customHeight="1" s="89">
       <c r="B37" s="12" t="inlineStr">
@@ -4297,23 +4149,6 @@
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
       </c>
-      <c r="G37" s="16" t="inlineStr">
-        <is>
-          <t>1.1 Costo de operación de automóvil Limonal – Cañas
-1.2 Costo de operación de camioneta Limonal – Cañas
-1.3 Costo de operación de autobús Limonal – Cañas
-1.4 Costo de operación de camión C2 Limonal – Cañas
-1.5 Costo de operación de camión C3 Limonal – Cañas
-1.6 Costo de operación de camión articulado Limonal – Cañas
-2.1 Tiempo medio de viaje de automóvil Limonal – Cañas
-2.2 Tiempo medio de viaje de camioneta Limonal – Cañas
-2.3 Tiempo medio de viaje de autobús Limonal – Cañas
-2.4 Tiempo medio de viaje de camión C2 Limonal – Cañas
-2.5 Tiempo medio de viaje de camión C3 Limonal – Cañas
-2.6 Tiempo medio de viaje de camión articulado Limonal – Cañas
-3.2 Nivel de seguridad de la vía del tramo Limonal - Cañas</t>
-        </is>
-      </c>
     </row>
     <row r="38" ht="188.4" customHeight="1" s="89">
       <c r="B38" s="17" t="inlineStr">
@@ -4341,23 +4176,6 @@
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
       </c>
-      <c r="G38" s="20" t="inlineStr">
-        <is>
-          <t>1.7 Costo de operación de automóvil Playa Naranjo - Paquera
-1.8 Costo de operación de camioneta Playa Naranjo - Paquera
-1.9 Costo de operación de autobús Playa Naranjo - Paquera
-1.10 Costo de operación de camión C2 Playa Naranjo - Paquera
-1.11 Costo de operación de camión C3 Playa Naranjo - Paquera
-1.12 Costo de operación de camión articulado Playa Naranjo - Paquera
-2.7 Tiempo medio de viaje de automóvil Playa Naranjo - Paquera
-2.8 Tiempo medio de viaje de camioneta Playa Naranjo - Paquera
-2.9 Tiempo medio de viaje de autobús Playa Naranjo - Paquera
-2.10 Tiempo medio de viaje de camión C2 Playa Naranjo - Paquera
-2.11 Tiempo medio de viaje de camión C3 Playa Naranjo - Paquera
-2.12 Tiempo medio de viaje de camión articulado Playa Naranjo - Paquera
-3.3 Nivel de seguridad de la vía del tramo Playa Naranjo - Paquera</t>
-        </is>
-      </c>
     </row>
     <row r="39" ht="193.95" customHeight="1" s="89">
       <c r="B39" s="17" t="inlineStr">
@@ -4386,23 +4204,6 @@
 El plazo de ejecución de las obras supera el plazo actual del programa PIT</t>
         </is>
       </c>
-      <c r="G39" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.13 Costo de operación de automóvil Barranca - Limonal
-1.14 Costo de operación de camioneta Barranca - Limonal
-1.15 Costo de operación de autobús Barranca - Limonal
-1.16 Costo de operación de camión C2 Barranca - Limonal
-1.17 Costo de operación de camión C3 Barranca - Limonal
-1.18 Costo de operación de camión articulado Barranca - Limonal
-2.13 Tiempo medio de viaje de automóvil Barranca - Limonal
-2.14 Tiempo medio de viaje de camioneta Barranca - Limonal
-2.15 Tiempo medio de viaje de autobús Barranca - Limonal
-2.16 Tiempo medio de viaje de camión C2 Barranca - Limonal
-2.17 Tiempo medio de viaje de camión C3 Barranca - Limonal
-2.18 Tiempo medio de viaje de camión articulado Barranca - Limonal
-3.1 Nivel de seguridad de la vía del tramo Barranca Limonal </t>
-        </is>
-      </c>
     </row>
     <row r="40" ht="30.6" customHeight="1" s="89">
       <c r="B40" s="17" t="inlineStr">
@@ -4425,11 +4226,6 @@
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
       </c>
-      <c r="G40" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.4 Probabilidad de ocurrencia de una falla grave en el rompeolas del Puerto de Caldera </t>
-        </is>
-      </c>
     </row>
     <row r="41" ht="87" customHeight="1" s="89" thickBot="1">
       <c r="B41" s="27" t="inlineStr">
@@ -4451,13 +4247,6 @@
       <c r="F41" s="28" t="inlineStr">
         <is>
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
-        </is>
-      </c>
-      <c r="G41" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.5 Porcentaje de tiempo de operatividad de las terminales de transbordadores del Golfo de Nicoya 
-3.6 Aumento de satisfacción de usuarios de las terminales de Transbordadores (Hombres) 
-3.7 Aumento de satisfacción de usuarios de las terminales de Transbordadores (Mujeres) </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar hoja comentarios_clausulas y mostrarlos en cláusulas vencidas
- Nueva hoja 'comentarios_clausulas' en el Excel con columnas:
  Clause_ID, Fecha_Comentario, Autor, Comentario, Estado_Gestion, Fecha_Compromiso
  y validación de lista en Estado_Gestion (En gestión / Resuelto / Escalado)
- buildComentariosMap(): lee la hoja y devuelve el comentario más reciente por Clause_ID
- renderClausulasV(): reemplaza el guión vacío con el comentario real, badge de estado
  coloreado y fecha de compromiso si existe

https://claude.ai/code/session_01Vg346nWHMSdAxc2YdgMDKB
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -14,6 +14,7 @@
     <sheet name="resultados" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="productos_resultados" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="change log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="comentarios_clausulas" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'documentos'!$A$3:$D$60</definedName>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -190,8 +191,12 @@
       <color rgb="FF10B981"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -235,6 +240,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0F1825"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -561,7 +571,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -841,6 +851,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="8" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -13403,4 +13416,63 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="89" min="1" max="1"/>
+    <col width="18" customWidth="1" style="89" min="2" max="2"/>
+    <col width="20" customWidth="1" style="89" min="3" max="3"/>
+    <col width="60" customWidth="1" style="89" min="4" max="4"/>
+    <col width="18" customWidth="1" style="89" min="5" max="5"/>
+    <col width="18" customWidth="1" style="89" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="89">
+      <c r="A1" s="98" t="inlineStr">
+        <is>
+          <t>Clause_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="98" t="inlineStr">
+        <is>
+          <t>Fecha_Comentario</t>
+        </is>
+      </c>
+      <c r="C1" s="98" t="inlineStr">
+        <is>
+          <t>Autor</t>
+        </is>
+      </c>
+      <c r="D1" s="98" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="E1" s="98" t="inlineStr">
+        <is>
+          <t>Estado_Gestion</t>
+        </is>
+      </c>
+      <c r="F1" s="98" t="inlineStr">
+        <is>
+          <t>Fecha_Compromiso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor inválido" error="Use: En gestión, Resuelto o Escalado" type="list">
+      <formula1>"En gestión,Resuelto,Escalado"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Agregar comentarios a cláusulas vencidas 701558, 664364, 705320, 705321
Recordatorio enviado al jefe de equipo — autor: alvarobo, estado: En gestión,
fecha comentario: 2026-06-04, fecha compromiso: 2026-06-05

https://claude.ai/code/session_01Vg346nWHMSdAxc2YdgMDKB
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -28,7 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="26">
     <font>
       <name val="Aptos Narrow"/>
@@ -571,7 +573,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -855,6 +857,7 @@
     <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13424,7 +13427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="89" min="1" max="1"/>
@@ -13467,6 +13470,118 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>701558</t>
+        </is>
+      </c>
+      <c r="B2" s="99" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>alvarobo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Recordatorio enviado al jefe de equipo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>En gestión</t>
+        </is>
+      </c>
+      <c r="F2" s="99" t="n">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>664364</t>
+        </is>
+      </c>
+      <c r="B3" s="99" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>alvarobo</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Recordatorio enviado al jefe de equipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>En gestión</t>
+        </is>
+      </c>
+      <c r="F3" s="99" t="n">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>705320</t>
+        </is>
+      </c>
+      <c r="B4" s="99" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>alvarobo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Recordatorio enviado al jefe de equipo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>En gestión</t>
+        </is>
+      </c>
+      <c r="F4" s="99" t="n">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>705321</t>
+        </is>
+      </c>
+      <c r="B5" s="99" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>alvarobo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Recordatorio enviado al jefe de equipo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>En gestión</t>
+        </is>
+      </c>
+      <c r="F5" s="99" t="n">
+        <v>46178</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor inválido" error="Use: En gestión, Resuelto o Escalado" type="list">

</xml_diff>

<commit_message>
actualizacion de links de documentos
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\torre-control-ccr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/alvarobo_iadb_org/Documents/Documents/GitHub/torre-control-ccr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7705C02E-E2E5-42A1-8E9F-511396BD8ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{7705C02E-E2E5-42A1-8E9F-511396BD8ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{845FB217-8908-434E-A051-6BC21CA263FC}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="3000" windowWidth="23340" windowHeight="11295" tabRatio="819" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="documentos" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2152" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="676">
   <si>
     <t>Fecha de revisión</t>
   </si>
@@ -2098,6 +2098,24 @@
   </si>
   <si>
     <t>705321</t>
+  </si>
+  <si>
+    <t>https://ezws.iadb.org/getdocument.aspx?docnum=EZIDB0000195-246772048-17</t>
+  </si>
+  <si>
+    <t>EZIDB0000195-246772048-17</t>
+  </si>
+  <si>
+    <t>LP - Modification</t>
+  </si>
+  <si>
+    <t>LC - Loan modification</t>
+  </si>
+  <si>
+    <t>https://ezws.iadb.org/getdocument.aspx?docnum=EZIDB0000195-246772048-14</t>
+  </si>
+  <si>
+    <t>EZIDB0000195-246772048-14</t>
   </si>
 </sst>
 </file>
@@ -2862,6 +2880,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2876,15 +2898,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3216,8 +3234,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D62"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="61" customWidth="1"/>
     <col min="2" max="2" width="38" style="61" customWidth="1"/>
@@ -3228,12 +3246,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="93" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
     </row>
     <row r="2" spans="1:4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4044,6 +4062,34 @@
       </c>
       <c r="D60" s="63" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61" s="63" t="s">
+        <v>672</v>
+      </c>
+      <c r="C61" s="63" t="s">
+        <v>671</v>
+      </c>
+      <c r="D61" s="63" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="B62" s="63" t="s">
+        <v>673</v>
+      </c>
+      <c r="C62" s="63" t="s">
+        <v>675</v>
+      </c>
+      <c r="D62" s="63" t="s">
+        <v>674</v>
       </c>
     </row>
   </sheetData>
@@ -4058,7 +4104,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.5703125" customWidth="1"/>
     <col min="3" max="3" width="35.5703125" bestFit="1" customWidth="1"/>
@@ -4548,7 +4594,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:G70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" customWidth="1"/>
@@ -5089,7 +5135,7 @@
       <c r="E34" s="79" t="s">
         <v>316</v>
       </c>
-      <c r="F34" s="93" t="s">
+      <c r="F34" s="95" t="s">
         <v>314</v>
       </c>
       <c r="G34" s="80" t="s">
@@ -5109,7 +5155,7 @@
       <c r="E35" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="F35" s="94" t="s">
+      <c r="F35" s="96" t="s">
         <v>320</v>
       </c>
       <c r="G35" s="20" t="s">
@@ -5129,7 +5175,7 @@
       <c r="E36" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="F36" s="94" t="s">
+      <c r="F36" s="96" t="s">
         <v>324</v>
       </c>
       <c r="G36" s="20" t="s">
@@ -5673,7 +5719,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:Q14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="57.140625" customWidth="1"/>
@@ -6115,7 +6161,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -6261,7 +6307,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H113"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6273,16 +6319,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
         <v>440</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
     </row>
     <row r="2" spans="1:8" ht="4.9000000000000004" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9183,18 +9229,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C179"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="65" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
         <v>650</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
     </row>
     <row r="2" spans="1:3" ht="4.9000000000000004" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11156,7 +11202,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3768BFDA-6D4B-4C12-8BA7-7E70B4D9D70D}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -11166,22 +11212,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="89" t="s">
         <v>657</v>
       </c>
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="89" t="s">
         <v>658</v>
       </c>
-      <c r="C1" s="95" t="s">
+      <c r="C1" s="89" t="s">
         <v>659</v>
       </c>
-      <c r="D1" s="95" t="s">
+      <c r="D1" s="89" t="s">
         <v>660</v>
       </c>
-      <c r="E1" s="95" t="s">
+      <c r="E1" s="89" t="s">
         <v>661</v>
       </c>
-      <c r="F1" s="95" t="s">
+      <c r="F1" s="89" t="s">
         <v>662</v>
       </c>
     </row>
@@ -11189,7 +11235,7 @@
       <c r="A2" t="s">
         <v>663</v>
       </c>
-      <c r="B2" s="96">
+      <c r="B2" s="90">
         <v>46177</v>
       </c>
       <c r="C2" t="s">
@@ -11201,7 +11247,7 @@
       <c r="E2" t="s">
         <v>666</v>
       </c>
-      <c r="F2" s="96">
+      <c r="F2" s="90">
         <v>46178</v>
       </c>
     </row>
@@ -11209,7 +11255,7 @@
       <c r="A3" t="s">
         <v>667</v>
       </c>
-      <c r="B3" s="96">
+      <c r="B3" s="90">
         <v>46177</v>
       </c>
       <c r="C3" t="s">
@@ -11221,7 +11267,7 @@
       <c r="E3" t="s">
         <v>666</v>
       </c>
-      <c r="F3" s="96">
+      <c r="F3" s="90">
         <v>46178</v>
       </c>
     </row>
@@ -11229,7 +11275,7 @@
       <c r="A4" t="s">
         <v>668</v>
       </c>
-      <c r="B4" s="96">
+      <c r="B4" s="90">
         <v>46177</v>
       </c>
       <c r="C4" t="s">
@@ -11241,7 +11287,7 @@
       <c r="E4" t="s">
         <v>666</v>
       </c>
-      <c r="F4" s="96">
+      <c r="F4" s="90">
         <v>46178</v>
       </c>
     </row>
@@ -11249,7 +11295,7 @@
       <c r="A5" t="s">
         <v>669</v>
       </c>
-      <c r="B5" s="96">
+      <c r="B5" s="90">
         <v>46177</v>
       </c>
       <c r="C5" t="s">
@@ -11261,7 +11307,7 @@
       <c r="E5" t="s">
         <v>666</v>
       </c>
-      <c r="F5" s="96">
+      <c r="F5" s="90">
         <v>46178</v>
       </c>
     </row>
@@ -11278,7 +11324,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="B2:E51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Agrega columna Adquisicion_Critica a productos_adquisiciones
Permite marcar cuáles de las adquisiciones asociadas a un producto crítico
deben mostrarse en el tab (Sí/No). Las 7 filas existentes de CR-L1157 se
marcan como Sí por defecto. Se agrega entrada en change log.
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -2483,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E61"/>
+  <dimension ref="B2:E62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="3.7109375" customWidth="1" style="77" min="1" max="1"/>
@@ -3669,6 +3669,26 @@
       <c r="E61" t="inlineStr">
         <is>
           <t>Se agrega hoja productos_adquisiciones (relación Producto Crítico ↔ ID de Proceso) para permitir mostrar el nombre y detalle (monto, estado, método) de la adquisición crítica asociada a cada producto crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="68" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>productos_adquisiciones</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CR-L1157</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Se agrega columna Adquisicion_Critica (Sí/No) para que el tab de productos críticos pueda filtrar y mostrar solo las adquisiciones marcadas como críticas; las 7 filas existentes se marcan como Sí</t>
         </is>
       </c>
     </row>
@@ -14251,12 +14271,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="77" min="1" max="1"/>
     <col width="38" customWidth="1" style="77" min="2" max="2"/>
     <col width="22" customWidth="1" style="77" min="3" max="3"/>
+    <col width="16" customWidth="1" style="77" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28.15" customHeight="1" s="77">
@@ -14282,6 +14303,11 @@
           <t>ID_Proceso</t>
         </is>
       </c>
+      <c r="D3" s="78" t="inlineStr">
+        <is>
+          <t>Adquisicion_Critica</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14299,6 +14325,11 @@
           <t>CR-L1157-P00001</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14316,6 +14347,11 @@
           <t>CR-L1157-P00002-AA</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14333,6 +14369,11 @@
           <t>CR-L1157-P00005</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14350,6 +14391,11 @@
           <t>CR-L1157-P00003-AA</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14367,6 +14413,11 @@
           <t>CR-L1157-P00004</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14384,6 +14435,11 @@
           <t>CR-L1157-P00006</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14401,10 +14457,15 @@
           <t>CR-L1157-P00007</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega columna Riesgos_Comentarios a productos_adquisiciones
Mueve el riesgo/comentario a nivel de adquisición en vez de producto crítico,
ya que un producto puede tener varias adquisiciones críticas y cada una puede
tener su propio riesgo. Columna vacía por ahora, pendiente de que el equipo
del proyecto la llene. Se agrega entrada en change log.
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -2483,7 +2483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E62"/>
+  <dimension ref="B2:E63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="3.7109375" customWidth="1" style="77" min="1" max="1"/>
@@ -3689,6 +3689,26 @@
       <c r="E62" t="inlineStr">
         <is>
           <t>Se agrega columna Adquisicion_Critica (Sí/No) para que el tab de productos críticos pueda filtrar y mostrar solo las adquisiciones marcadas como críticas; las 7 filas existentes se marcan como Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="68" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>productos_adquisiciones</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CR-L1157</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Se agrega columna Riesgos_Comentarios para asociar el riesgo/comentario a cada adquisición crítica en vez de al producto crítico completo (columna vacía, pendiente de que el equipo del proyecto la llene por adquisición)</t>
         </is>
       </c>
     </row>
@@ -14271,13 +14291,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="77" min="1" max="1"/>
     <col width="38" customWidth="1" style="77" min="2" max="2"/>
     <col width="22" customWidth="1" style="77" min="3" max="3"/>
     <col width="16" customWidth="1" style="77" min="4" max="4"/>
+    <col width="40" customWidth="1" style="77" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28.15" customHeight="1" s="77">
@@ -14308,6 +14329,11 @@
           <t>Adquisicion_Critica</t>
         </is>
       </c>
+      <c r="E3" s="78" t="inlineStr">
+        <is>
+          <t>Riesgos_Comentarios</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14465,7 +14491,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega Intercambio San Ramón/Grecia y elimina producto de Supervisión (CR-L1139)
Se agregan 2 productos críticos faltantes en CR-L1139: "Intercambio de San
Ramón" e "Intercambio de Grecia" (Lote #4 OBIS), ambos con CR-L1139-P00045
como adquisición crítica (mismo contrato combinado de diseño+construcción
que ya cubre Naranjo, según el raw data).

Se elimina el producto crítico "Lote #4 OBIS – Supervisión D+C Intercambio
Coyol" de productos criticos y productos_adquisiciones. La adquisición de
supervisión CR-L1139-P00048 pasa a asociarse como "No" (no crítica) a los 4
productos de intercambio (Naranjo, Coyol, San Ramón, Grecia) en vez de tener
su propio producto crítico independiente.

Se agregan 2 entradas en change log.
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -432,7 +432,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -646,6 +646,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2483,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E68"/>
+  <dimension ref="B2:E70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="3.7109375" customWidth="1" style="77" min="1" max="1"/>
@@ -3809,6 +3819,46 @@
       <c r="E68" t="inlineStr">
         <is>
           <t>Se agregan 10 filas: relación producto crítico ↔ adquisición crítica (préstamo 5823/OC-CR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="68" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>productos criticos, productos_adquisiciones</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Se agregan los productos críticos faltantes 'Intercambio de San Ramón' e 'Intercambio de Grecia' (Lote #4 OBIS), con su adquisición crítica asociada CR-L1139-P00045 (mismo contrato combinado que ya cubre Naranjo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="68" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>productos criticos, productos_adquisiciones</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Se elimina el producto crítico 'Lote #4 OBIS – Supervisión D+C Intercambio Coyol'. La adquisición de supervisión CR-L1139-P00048 pasa a asociarse como 'No' (no crítica) a los 4 productos de intercambio (Naranjo, Coyol, San Ramón, Grecia) en vez de tener su propio producto crítico.</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F70"/>
+  <dimension ref="A2:F71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" style="74" min="1" max="1"/>
@@ -5442,127 +5492,114 @@
       <c r="F36" s="75" t="n"/>
     </row>
     <row r="37" ht="45" customHeight="1" s="77">
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="79" t="inlineStr">
         <is>
           <t>CR-L1139</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>Lote #4 OBIS – Supervisión D+C Intercambio Coyol</t>
-        </is>
-      </c>
-      <c r="D37" s="74" t="inlineStr">
+      <c r="C37" s="80" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de San Ramón</t>
+        </is>
+      </c>
+      <c r="D37" s="81" t="inlineStr">
+        <is>
+          <t>En tiempo</t>
+        </is>
+      </c>
+      <c r="E37" s="81" t="n"/>
+      <c r="F37" s="82" t="n"/>
+    </row>
+    <row r="38" ht="30.75" customHeight="1" s="77" thickBot="1">
+      <c r="B38" s="79" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="C38" s="80" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de Grecia</t>
+        </is>
+      </c>
+      <c r="D38" s="81" t="inlineStr">
+        <is>
+          <t>En tiempo</t>
+        </is>
+      </c>
+      <c r="E38" s="81" t="n"/>
+      <c r="F38" s="82" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="77" thickBot="1">
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados</t>
+        </is>
+      </c>
+      <c r="D39" s="74" t="inlineStr">
         <is>
           <t>Retrasado</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
-        <is>
-          <t>Supervisión D+C Intercambio Coyol
-(firma consultora)</t>
-        </is>
-      </c>
-      <c r="F37" s="15" t="inlineStr">
-        <is>
-          <t>NOB condicionada a ajustes al documento de SDP.
-Estimado por US$2.5 millones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30.75" customHeight="1" s="77" thickBot="1">
-      <c r="B38" s="14" t="inlineStr">
+      <c r="E39" s="74" t="inlineStr">
+        <is>
+          <t>Estructuración APP #2</t>
+        </is>
+      </c>
+      <c r="F39" s="74" t="inlineStr">
+        <is>
+          <t>Proyecto #2 aún no definido por el OE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="120" customHeight="1" s="77">
+      <c r="B40" s="64" t="inlineStr">
         <is>
           <t>CR-L1139</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
-        <is>
-          <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados</t>
-        </is>
-      </c>
-      <c r="D38" s="74" t="inlineStr">
+      <c r="C40" s="65" t="inlineStr">
+        <is>
+          <t>Intercambios Taras – La Lima construidos</t>
+        </is>
+      </c>
+      <c r="D40" s="66" t="inlineStr">
         <is>
           <t>Retrasado</t>
         </is>
       </c>
-      <c r="E38" s="74" t="inlineStr">
-        <is>
-          <t>Estructuración APP #2</t>
-        </is>
-      </c>
-      <c r="F38" s="74" t="inlineStr">
-        <is>
-          <t>Proyecto #2 aún no definido por el OE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1" s="77" thickBot="1">
-      <c r="B39" s="64" t="inlineStr">
-        <is>
-          <t>CR-L1139</t>
-        </is>
-      </c>
-      <c r="C39" s="65" t="inlineStr">
-        <is>
-          <t>Intercambios Taras – La Lima construidos</t>
-        </is>
-      </c>
-      <c r="D39" s="66" t="inlineStr">
-        <is>
-          <t>Retrasado</t>
-        </is>
-      </c>
-      <c r="E39" s="66" t="n"/>
-      <c r="F39" s="66" t="n"/>
-    </row>
-    <row r="40" ht="120" customHeight="1" s="77">
-      <c r="B40" s="11" t="inlineStr">
+      <c r="E40" s="66" t="n"/>
+      <c r="F40" s="66" t="n"/>
+    </row>
+    <row r="41" ht="45" customHeight="1" s="77">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>CR-G1008</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable
 1.2 Número total de espacios públicos que disponen de sistema saneamiento nuevos o mejorados</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>En tiempo</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Consultoría Diagnóstico para identificación y selección de necesidades de sistemas de saneamiento y capacitación a usuarios del sistema/  Diagnóstico para idenficar  hogares y principales barreras para su conectividad  a los servicios de los acueductos beneficiados por el PAPS. </t>
         </is>
       </c>
-      <c r="F40" s="12" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Se debe actualizar la planificación para validarla mediante un taller de arranque, junto con la Unidad Ejecutora y la Jefe de Equipo. </t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="45" customHeight="1" s="77">
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>CR-G1008</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable</t>
-        </is>
-      </c>
-      <c r="D41" s="74" t="inlineStr">
-        <is>
-          <t>En tiempo</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>Diseño de la obra e inspección (sistemas de saneamiento).</t>
         </is>
       </c>
     </row>
@@ -5584,59 +5621,54 @@
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
+          <t>Diseño de la obra e inspección (sistemas de saneamiento).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1" s="77">
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>CR-G1008</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>1.1 Número total de hogares que disponen de sistema de saneamiento nuevo o mejorado y/o conexión al agua potable</t>
+        </is>
+      </c>
+      <c r="D43" s="74" t="inlineStr">
+        <is>
+          <t>En tiempo</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
           <t>Sistemas de Saneamiento en hogares rurales (construcción de la obra)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="45" customHeight="1" s="77">
-      <c r="B43" s="11" t="inlineStr">
+    <row r="44" ht="45" customHeight="1" s="77">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>CR-L1032</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>Tramo Limonal - Cañas rehabilitado y ampliado</t>
         </is>
       </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>Logrado</t>
         </is>
       </c>
-      <c r="E43" s="12" t="inlineStr">
+      <c r="E44" s="12" t="inlineStr">
         <is>
           <t>Construcción de la Ampliación y Rehabilitación del Tramo de Carretera Limonal-Cañas</t>
         </is>
       </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="45" customHeight="1" s="77">
-      <c r="B44" s="14" t="inlineStr">
-        <is>
-          <t>CR-L1032</t>
-        </is>
-      </c>
-      <c r="C44" s="74" t="inlineStr">
-        <is>
-          <t>Tramo Playa Naranjo - Paquera rehabilitado y ampliado</t>
-        </is>
-      </c>
-      <c r="D44" s="74" t="inlineStr">
-        <is>
-          <t>Logrado</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>Construcción de la Ampliación y Rehabilitación del Tramo de Carretera Playa Naranjo – Paquera RN 160</t>
-        </is>
-      </c>
-      <c r="F44" s="15" t="inlineStr">
+      <c r="F44" s="12" t="inlineStr">
         <is>
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
@@ -5650,89 +5682,97 @@
       </c>
       <c r="C45" s="74" t="inlineStr">
         <is>
+          <t>Tramo Playa Naranjo - Paquera rehabilitado y ampliado</t>
+        </is>
+      </c>
+      <c r="D45" s="74" t="inlineStr">
+        <is>
+          <t>Logrado</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>Construcción de la Ampliación y Rehabilitación del Tramo de Carretera Playa Naranjo – Paquera RN 160</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45" customHeight="1" s="77">
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>CR-L1032</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
           <t>Tramo Barranca-Limonal rehabilitado y ampliado</t>
         </is>
       </c>
-      <c r="D45" s="74" t="inlineStr">
+      <c r="D46" s="74" t="inlineStr">
         <is>
           <t>Retrasado</t>
         </is>
       </c>
-      <c r="E45" s="15" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>Rehabilitación y ampliación a cuatro carriles de la Ruta Nacional No. 1, Sección Barranca – Limonal (SICOP 2025LY-00001-0003000001)</t>
         </is>
       </c>
-      <c r="F45" s="15" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
         <is>
           <t>La unidad ejecutora no tiene responsabilidad directa sobre el proceso al estar a cargo de CONAVI con contrapartida
 El plazo de ejecución de las obras supera el plazo actual del programa PIT</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="45" customHeight="1" s="77">
-      <c r="B46" s="14" t="inlineStr">
+    <row r="47" ht="45.75" customHeight="1" s="77" thickBot="1">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>CR-L1032</t>
         </is>
       </c>
-      <c r="C46" s="74" t="inlineStr">
+      <c r="C47" s="74" t="inlineStr">
         <is>
           <t>Rompeolas de Caldera rehabilitado y ampliado</t>
         </is>
       </c>
-      <c r="D46" s="74" t="inlineStr">
+      <c r="D47" s="74" t="inlineStr">
         <is>
           <t>Logrado</t>
         </is>
       </c>
-      <c r="F46" s="15" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="45.75" customHeight="1" s="77" thickBot="1">
-      <c r="B47" s="19" t="inlineStr">
+    <row r="48" ht="45.75" customHeight="1" s="77" thickBot="1">
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>CR-L1032</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>Terminales de transbordadores rehabilitadas</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>Logrado</t>
         </is>
       </c>
-      <c r="E47" s="21" t="n"/>
-      <c r="F47" s="20" t="inlineStr">
+      <c r="E48" s="21" t="n"/>
+      <c r="F48" s="20" t="inlineStr">
         <is>
           <t>Evaluación de resultados pendiente para confirmar cumplimiento de indicadores</t>
         </is>
       </c>
-    </row>
-    <row r="48" ht="45.75" customHeight="1" s="77" thickBot="1">
-      <c r="B48" s="64" t="inlineStr">
-        <is>
-          <t>CR-L1152</t>
-        </is>
-      </c>
-      <c r="C48" s="65" t="inlineStr">
-        <is>
-          <t>Centros educativos priorizados con programas de clima escolar con enfoque en diversidad implementados</t>
-        </is>
-      </c>
-      <c r="D48" s="66" t="inlineStr">
-        <is>
-          <t>En tiempo</t>
-        </is>
-      </c>
-      <c r="E48" s="66" t="n"/>
-      <c r="F48" s="66" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="77" thickBot="1">
       <c r="B49" s="64" t="inlineStr">
@@ -5742,7 +5782,7 @@
       </c>
       <c r="C49" s="65" t="inlineStr">
         <is>
-          <t>Computadoras personales entregadas</t>
+          <t>Centros educativos priorizados con programas de clima escolar con enfoque en diversidad implementados</t>
         </is>
       </c>
       <c r="D49" s="66" t="inlineStr">
@@ -5761,7 +5801,7 @@
       </c>
       <c r="C50" s="65" t="inlineStr">
         <is>
-          <t>Cupos abiertos al personal educativo de cursos de formación para el desarrollo de competencias</t>
+          <t>Computadoras personales entregadas</t>
         </is>
       </c>
       <c r="D50" s="66" t="inlineStr">
@@ -5780,7 +5820,7 @@
       </c>
       <c r="C51" s="65" t="inlineStr">
         <is>
-          <t>Equipos tecnológicos educativos de aula y para los estudiantes con criterios de eficiencia entregados a los Centros Educativos</t>
+          <t>Cupos abiertos al personal educativo de cursos de formación para el desarrollo de competencias</t>
         </is>
       </c>
       <c r="D51" s="66" t="inlineStr">
@@ -5799,7 +5839,7 @@
       </c>
       <c r="C52" s="65" t="inlineStr">
         <is>
-          <t>Estudios de grabación con equipamiento para la producción de materiales didácticos mejorados</t>
+          <t>Equipos tecnológicos educativos de aula y para los estudiantes con criterios de eficiencia entregados a los Centros Educativos</t>
         </is>
       </c>
       <c r="D52" s="66" t="inlineStr">
@@ -5818,7 +5858,7 @@
       </c>
       <c r="C53" s="65" t="inlineStr">
         <is>
-          <t>Informes sobre Autoevaluaciones docentes desarrolladas e implementadas</t>
+          <t>Estudios de grabación con equipamiento para la producción de materiales didácticos mejorados</t>
         </is>
       </c>
       <c r="D53" s="66" t="inlineStr">
@@ -5837,7 +5877,7 @@
       </c>
       <c r="C54" s="65" t="inlineStr">
         <is>
-          <t>Juntas Escolares y Administrativas que reciben asistencia técnica al menos una vez cada dos meses</t>
+          <t>Informes sobre Autoevaluaciones docentes desarrolladas e implementadas</t>
         </is>
       </c>
       <c r="D54" s="66" t="inlineStr">
@@ -5856,7 +5896,7 @@
       </c>
       <c r="C55" s="65" t="inlineStr">
         <is>
-          <t>Paquetes de Libros de texto y cuadernos de estudiante</t>
+          <t>Juntas Escolares y Administrativas que reciben asistencia técnica al menos una vez cada dos meses</t>
         </is>
       </c>
       <c r="D55" s="66" t="inlineStr">
@@ -5875,7 +5915,7 @@
       </c>
       <c r="C56" s="65" t="inlineStr">
         <is>
-          <t>Plataforma para el Sistema de gestión de Juntas Escolares y Administrativas, en funcionamiento</t>
+          <t>Paquetes de Libros de texto y cuadernos de estudiante</t>
         </is>
       </c>
       <c r="D56" s="66" t="inlineStr">
@@ -5894,7 +5934,7 @@
       </c>
       <c r="C57" s="65" t="inlineStr">
         <is>
-          <t>Plataformas educativas desarrolladas con enfoque de género y diversidad para estudiantes y docentes con catálogo y repositorio de recursos digitales por competencias</t>
+          <t>Plataforma para el Sistema de gestión de Juntas Escolares y Administrativas, en funcionamiento</t>
         </is>
       </c>
       <c r="D57" s="66" t="inlineStr">
@@ -5913,7 +5953,7 @@
       </c>
       <c r="C58" s="65" t="inlineStr">
         <is>
-          <t>Reportes de actualización de Programas de Estudios (primera infancia, primaria, secundaria y educación de jóvenes y adultos) con enfoque por competencias aprobados</t>
+          <t>Plataformas educativas desarrolladas con enfoque de género y diversidad para estudiantes y docentes con catálogo y repositorio de recursos digitales por competencias</t>
         </is>
       </c>
       <c r="D58" s="66" t="inlineStr">
@@ -5932,7 +5972,7 @@
       </c>
       <c r="C59" s="65" t="inlineStr">
         <is>
-          <t>Servicios de implementación de Planes de Recuperación de Aprendizajes (PRA) para centros educativos priorizados de primaria y secundaria entregados</t>
+          <t>Reportes de actualización de Programas de Estudios (primera infancia, primaria, secundaria y educación de jóvenes y adultos) con enfoque por competencias aprobados</t>
         </is>
       </c>
       <c r="D59" s="66" t="inlineStr">
@@ -5951,7 +5991,7 @@
       </c>
       <c r="C60" s="65" t="inlineStr">
         <is>
-          <t>Servicios individuales de tutorías remotas en funcionamiento</t>
+          <t>Servicios de implementación de Planes de Recuperación de Aprendizajes (PRA) para centros educativos priorizados de primaria y secundaria entregados</t>
         </is>
       </c>
       <c r="D60" s="66" t="inlineStr">
@@ -5965,12 +6005,12 @@
     <row r="61" ht="30.75" customHeight="1" s="77" thickBot="1">
       <c r="B61" s="64" t="inlineStr">
         <is>
-          <t>CR-L1156</t>
+          <t>CR-L1152</t>
         </is>
       </c>
       <c r="C61" s="65" t="inlineStr">
         <is>
-          <t>Modelo de fiscalización de la calidad de servicios en las Organizaciones de Bienestar Social</t>
+          <t>Servicios individuales de tutorías remotas en funcionamiento</t>
         </is>
       </c>
       <c r="D61" s="66" t="inlineStr">
@@ -5989,7 +6029,7 @@
       </c>
       <c r="C62" s="65" t="inlineStr">
         <is>
-          <t>Modelo de focalización con línea de pobreza ajustada por discapacidad y dependencia</t>
+          <t>Modelo de fiscalización de la calidad de servicios en las Organizaciones de Bienestar Social</t>
         </is>
       </c>
       <c r="D62" s="66" t="inlineStr">
@@ -6008,7 +6048,7 @@
       </c>
       <c r="C63" s="65" t="inlineStr">
         <is>
-          <t>Plataforma de vinculación de usuarios de servicios de cuidados y personas cuidadoras (CUIDAR.CR)</t>
+          <t>Modelo de focalización con línea de pobreza ajustada por discapacidad y dependencia</t>
         </is>
       </c>
       <c r="D63" s="66" t="inlineStr">
@@ -6027,7 +6067,7 @@
       </c>
       <c r="C64" s="65" t="inlineStr">
         <is>
-          <t>Registro Nacional de Personas Cuidadoras con código QR en CUIDAR.CR</t>
+          <t>Plataforma de vinculación de usuarios de servicios de cuidados y personas cuidadoras (CUIDAR.CR)</t>
         </is>
       </c>
       <c r="D64" s="66" t="inlineStr">
@@ -6046,7 +6086,7 @@
       </c>
       <c r="C65" s="65" t="inlineStr">
         <is>
-          <t>Sistema de valoración funcional de la dependencia</t>
+          <t>Registro Nacional de Personas Cuidadoras con código QR en CUIDAR.CR</t>
         </is>
       </c>
       <c r="D65" s="66" t="inlineStr">
@@ -6065,7 +6105,7 @@
       </c>
       <c r="C66" s="65" t="inlineStr">
         <is>
-          <t>Ventanilla Única de Servicios con baremo incorporado al sistema de referencias del SINIRUBE</t>
+          <t>Sistema de valoración funcional de la dependencia</t>
         </is>
       </c>
       <c r="D66" s="66" t="inlineStr">
@@ -6079,12 +6119,12 @@
     <row r="67" ht="15.75" customHeight="1" s="77" thickBot="1">
       <c r="B67" s="64" t="inlineStr">
         <is>
-          <t>CR-L1157</t>
+          <t>CR-L1156</t>
         </is>
       </c>
       <c r="C67" s="65" t="inlineStr">
         <is>
-          <t>Casa de máquinas modernizada</t>
+          <t>Ventanilla Única de Servicios con baremo incorporado al sistema de referencias del SINIRUBE</t>
         </is>
       </c>
       <c r="D67" s="66" t="inlineStr">
@@ -6103,7 +6143,7 @@
       </c>
       <c r="C68" s="65" t="inlineStr">
         <is>
-          <t>Luminarias LED instaladas</t>
+          <t>Casa de máquinas modernizada</t>
         </is>
       </c>
       <c r="D68" s="66" t="inlineStr">
@@ -6122,7 +6162,7 @@
       </c>
       <c r="C69" s="65" t="inlineStr">
         <is>
-          <t>Obras de captación de agua modernizadas</t>
+          <t>Luminarias LED instaladas</t>
         </is>
       </c>
       <c r="D69" s="66" t="inlineStr">
@@ -6141,16 +6181,35 @@
       </c>
       <c r="C70" s="65" t="inlineStr">
         <is>
-          <t>Transformadores de potencia y reactores instalados</t>
+          <t>Obras de captación de agua modernizadas</t>
         </is>
       </c>
       <c r="D70" s="66" t="inlineStr">
         <is>
-          <t>Pausado</t>
+          <t>En tiempo</t>
         </is>
       </c>
       <c r="E70" s="66" t="n"/>
       <c r="F70" s="66" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="64" t="inlineStr">
+        <is>
+          <t>CR-L1157</t>
+        </is>
+      </c>
+      <c r="C71" s="65" t="inlineStr">
+        <is>
+          <t>Transformadores de potencia y reactores instalados</t>
+        </is>
+      </c>
+      <c r="D71" s="66" t="inlineStr">
+        <is>
+          <t>Pausado</t>
+        </is>
+      </c>
+      <c r="E71" s="66" t="n"/>
+      <c r="F71" s="66" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B3:F34"/>
@@ -14391,7 +14450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="77" min="1" max="1"/>
@@ -15067,118 +15126,111 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="78" t="inlineStr">
         <is>
           <t>CR-L1139</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Lote #4 OBIS – Supervisión D+C Intercambio Coyol</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B32" s="78" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de San Ramón</t>
+        </is>
+      </c>
+      <c r="C32" s="78" t="inlineStr">
+        <is>
+          <t>CR-L1139-P00045</t>
+        </is>
+      </c>
+      <c r="D32" s="78" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E32" s="78" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="78" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="B33" s="78" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de San Ramón</t>
+        </is>
+      </c>
+      <c r="C33" s="78" t="inlineStr">
         <is>
           <t>CR-L1139-P00048</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" s="78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E33" s="78" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="78" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="B34" s="78" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de Grecia</t>
+        </is>
+      </c>
+      <c r="C34" s="78" t="inlineStr">
+        <is>
+          <t>CR-L1139-P00045</t>
+        </is>
+      </c>
+      <c r="D34" s="78" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>NOB condicionada a ajustes al documento de SDP.
-Estimado por US$2.5 millones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="E34" s="78" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="78" t="inlineStr">
         <is>
           <t>CR-L1139</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>CR-L1139-P00024</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Proyecto #2 aún no definido por el OE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>CR-L1139</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Intercambios Taras – La Lima construidos</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>CR-L1139-P00001</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>CR-L1139</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Intercambios Taras – La Lima construidos</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CR-L1139-P00008</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="B35" s="78" t="inlineStr">
+        <is>
+          <t>Lote #4 OBIS corredor San Ramón–San José: Intercambio de Grecia</t>
+        </is>
+      </c>
+      <c r="C35" s="78" t="inlineStr">
+        <is>
+          <t>CR-L1139-P00048</t>
+        </is>
+      </c>
+      <c r="D35" s="78" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="E35" s="78" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CR-L1137</t>
+          <t>CR-L1139</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Delegaciones diseñadas, construidas, equipadas y operando bajo enfoque de policía comunitaria</t>
+          <t>Estudios de Estructuración integral en al menos dos proyectos APP realizados</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CR-L1137-P00367</t>
+          <t>CR-L1139-P00024</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -15188,61 +15240,51 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
+          <t>Proyecto #2 aún no definido por el OE.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CR-L1137</t>
+          <t>CR-L1139</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Delegaciones diseñadas, construidas, equipadas y operando bajo enfoque de policía comunitaria</t>
+          <t>Intercambios Taras – La Lima construidos</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CR-L1137-P00375</t>
+          <t>CR-L1139-P00001</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>Sí</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CR-L1137</t>
+          <t>CR-L1139</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Centro de Mando y Control Policial construido, equipado y en funcionamiento</t>
+          <t>Intercambios Taras – La Lima construidos</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CR-L1137-P00348</t>
+          <t>CR-L1139-P00008</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa.</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -15254,17 +15296,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Estrategia de comunicación social de los CCP diseñada e implementada</t>
+          <t>Delegaciones diseñadas, construidas, equipadas y operando bajo enfoque de policía comunitaria</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CR-L1137-P00253</t>
+          <t>CR-L1137-P00367</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
@@ -15276,17 +15323,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Municipalidades y grupos de sociedad civil capacitados en prevención de violencia</t>
+          <t>Delegaciones diseñadas, construidas, equipadas y operando bajo enfoque de policía comunitaria</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CR-L1137-P00198</t>
+          <t>CR-L1137-P00375</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
@@ -15298,12 +15350,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
+          <t>Centro de Mando y Control Policial construido, equipado y en funcionamiento</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CR-L1137-P00326</t>
+          <t>CR-L1137-P00348</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -15313,7 +15365,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
+          <t>Adenda para incorporar equipo tecnológico tiene un plazo de ejecución cercano a la finalización del programa.</t>
         </is>
       </c>
     </row>
@@ -15325,22 +15377,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
+          <t>Estrategia de comunicación social de los CCP diseñada e implementada</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CR-L1137-P00327</t>
+          <t>CR-L1137-P00253</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>Sí</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
     </row>
@@ -15352,22 +15399,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
+          <t>Municipalidades y grupos de sociedad civil capacitados en prevención de violencia</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CR-L1137-P00347</t>
+          <t>CR-L1137-P00198</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Sí</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
     </row>
@@ -15379,34 +15421,39 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Modelo de gestión y atención de los CCP homologado, fortalecido y en funcionamiento</t>
+          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CR-L1137-P00314</t>
+          <t>CR-L1137-P00326</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CR-J0002</t>
+          <t>CR-L1137</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Unidad de refugio construida, equipada y en funcionamiento</t>
+          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CR-J0002-P00189</t>
+          <t>CR-L1137-P00327</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -15416,24 +15463,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CR-J0002</t>
+          <t>CR-L1137</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Campaña de comunicación contra la xenofobia realizada</t>
+          <t>Centros Cívicos diseñados, construidos, equipados y operando</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CR-J0002-P00240</t>
+          <t>CR-L1137-P00347</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -15443,34 +15490,29 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>El proceso de adquisición no ha iniciado</t>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos. Avance físico limitado con riesgo de finalizar con retraso.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CR-J0002</t>
+          <t>CR-L1137</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Centro Cívico de Upala construido, equipado y en funcionamiento</t>
+          <t>Modelo de gestión y atención de los CCP homologado, fortalecido y en funcionamiento</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CR-J0002-P00187</t>
+          <t>CR-L1137-P00314</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>Sí</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
@@ -15482,17 +15524,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
+          <t>Unidad de refugio construida, equipada y en funcionamiento</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CR-J0002-P00041</t>
+          <t>CR-J0002-P00189</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
@@ -15504,17 +15551,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
+          <t>Campaña de comunicación contra la xenofobia realizada</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CR-J0002-P00198</t>
+          <t>CR-J0002-P00240</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>El proceso de adquisición no ha iniciado</t>
         </is>
       </c>
     </row>
@@ -15526,17 +15578,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
+          <t>Centro Cívico de Upala construido, equipado y en funcionamiento</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CR-J0002-P00199</t>
+          <t>CR-J0002-P00187</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Procesos estimados para finalizar en 2027 cerca del fin del plazo de desembolsos</t>
         </is>
       </c>
     </row>
@@ -15548,12 +15605,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Procesos formativos para el fortalecimiento de los Centros Cívicos</t>
+          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CR-J0002-P00039</t>
+          <t>CR-J0002-P00041</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -15570,12 +15627,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Actualización de plataforma tecnológica de la DGME</t>
+          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CR-J0002-P00201</t>
+          <t>CR-J0002-P00198</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -15587,44 +15644,39 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CR-L1151</t>
+          <t>CR-J0002</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tramo Central Sifón – Sucre </t>
+          <t>Programas de formación para la prevención de la trata de personas y tráfico ilegal de migrantes</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CR-L1151-P00004</t>
+          <t>CR-J0002-P00199</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>Sí</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>En análisis por FMP y TSP junto con el OE sobre siguiente estado del proceso: declaración de infructuoso, cancelación, o nueva fuente de financiamiento.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CR-L1151</t>
+          <t>CR-J0002</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obras complementarias en el Tramo Central Sección Sucre – Abundancia </t>
+          <t>Procesos formativos para el fortalecimiento de los Centros Cívicos</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CR-L1151-P00004</t>
+          <t>CR-J0002-P00039</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -15636,97 +15688,102 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>CR-J0002</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Actualización de plataforma tecnológica de la DGME</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CR-J0002-P00201</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>CR-L1151</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tramo Central Sifón – Sucre </t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CR-L1151-P00004</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>En análisis por FMP y TSP junto con el OE sobre siguiente estado del proceso: declaración de infructuoso, cancelación, o nueva fuente de financiamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obras complementarias en el Tramo Central Sección Sucre – Abundancia </t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CR-L1151-P00004</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>Punta Sur de la RN-35 diseñado y construido</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>CR-L1151-P00003</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Lote 1 firmado
 Lote 2 firmado.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>CR-L1151</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Punta Sur de la RN-35 diseñado y construido</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>CR-L1151-P00010</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>CR-L1151</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>CR-L1151-P00001</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>CR-L1151</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>CR-L1151-P00002</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -15735,17 +15792,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Guía de indicadores mínimos para el monitoreo de la gestión de operación y mantenimiento del corredor RN-35</t>
+          <t>Punta Sur de la RN-35 diseñado y construido</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CR-L1151-P00007</t>
+          <t>CR-L1151-P00010</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -15757,12 +15814,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Plan de comunicación para promoción de prácticas seguras de conducción en el corredor</t>
+          <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CR-L1151-P00008</t>
+          <t>CR-L1151-P00001</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -15779,12 +15836,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Plan de mejora de las capacidades de gestión de riesgo de desastres y CC</t>
+          <t xml:space="preserve">Obras complementarias en la Punta Norte </t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CR-L1151-P00006</t>
+          <t>CR-L1151-P00002</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -15801,15 +15858,81 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>Guía de indicadores mínimos para el monitoreo de la gestión de operación y mantenimiento del corredor RN-35</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CR-L1151-P00007</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Plan de comunicación para promoción de prácticas seguras de conducción en el corredor</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CR-L1151-P00008</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Plan de mejora de las capacidades de gestión de riesgo de desastres y CC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CR-L1151-P00006</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>Programa de capacitación a funcionarios públicos para el diseño de pliegos con enfoque de género</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>CR-L1151-P00009</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>

</xml_diff>